<commit_message>
added catatan fields in claim preview window
</commit_message>
<xml_diff>
--- a/OTTimetableApp/Template/ot_template.xlsx
+++ b/OTTimetableApp/Template/ot_template.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="26327"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29725"/>
   <workbookPr updateLinks="always" codeName="ThisWorkbook" defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\PC\source\repos\OTTimetableApp\OTTimetableApp\Template\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\source\repos\OTTimetableApp\OTTimetableApp\Template\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C7FA7371-79C4-4341-A7D5-8808BC7EF150}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{42A87795-5ADA-44A3-9E43-EDC74F72EE02}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="5550" yWindow="1020" windowWidth="22500" windowHeight="11790" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Claim" sheetId="92" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="150" uniqueCount="114">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="148" uniqueCount="112">
   <si>
     <t>JABATAN KASTAM DIRAJA MALAYSIA</t>
   </si>
@@ -338,12 +338,6 @@
   </si>
   <si>
     <t xml:space="preserve">NO. KP   </t>
-  </si>
-  <si>
-    <t>MENYEMAK IMEJ/ MENAHAN KONTENA</t>
-  </si>
-  <si>
-    <t>Menyemak sistem SMK dan GCS, Menganalisa imej dagangan kontena dan menahan kontena</t>
   </si>
   <si>
     <t>SIJIL TUNTUTAN LEBIHMASA MENGIKUT SURAT</t>
@@ -2022,17 +2016,213 @@
     <xf numFmtId="0" fontId="43" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyProtection="1">
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="173" fontId="43" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="173" fontId="43" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="173" fontId="43" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="173" fontId="43" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="2" fontId="7" fillId="0" borderId="58" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="7" fillId="0" borderId="9" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="6" fillId="0" borderId="39" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="166" fontId="6" fillId="0" borderId="40" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="166" fontId="6" fillId="0" borderId="44" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="166" fontId="3" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="166" fontId="6" fillId="0" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="166" fontId="6" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="166" fontId="6" fillId="0" borderId="30" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="166" fontId="6" fillId="0" borderId="32" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="166" fontId="6" fillId="0" borderId="33" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="166" fontId="6" fillId="0" borderId="34" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="166" fontId="6" fillId="0" borderId="29" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="166" fontId="6" fillId="0" borderId="28" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="166" fontId="6" fillId="0" borderId="31" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="166" fontId="6" fillId="0" borderId="32" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="166" fontId="6" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="166" fontId="6" fillId="0" borderId="29" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="166" fontId="7" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="49" fontId="8" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="166" fontId="9" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="1" fontId="11" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="49" fontId="6" fillId="0" borderId="9" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="49" fontId="6" fillId="0" borderId="22" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="2" fontId="7" fillId="0" borderId="59" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="7" fillId="0" borderId="45" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="11" fillId="0" borderId="60" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="166" fontId="11" fillId="0" borderId="61" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="166" fontId="39" fillId="0" borderId="27" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="166" fontId="39" fillId="0" borderId="61" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="166" fontId="6" fillId="0" borderId="2" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="166" fontId="6" fillId="0" borderId="16" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="166" fontId="6" fillId="0" borderId="4" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="166" fontId="6" fillId="0" borderId="5" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="166" fontId="6" fillId="0" borderId="8" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="174" fontId="7" fillId="0" borderId="58" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="174" fontId="7" fillId="0" borderId="9" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="173" fontId="7" fillId="2" borderId="7" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="173" fontId="7" fillId="2" borderId="8" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
     </xf>
     <xf numFmtId="173" fontId="7" fillId="2" borderId="12" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -2042,11 +2232,176 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="173" fontId="7" fillId="2" borderId="7" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="173" fontId="43" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="173" fontId="43" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="173" fontId="43" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="173" fontId="43" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="36" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="173" fontId="7" fillId="2" borderId="8" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="169" fontId="13" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="166" fontId="12" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="37" fillId="0" borderId="0" xfId="0" applyFont="1" applyProtection="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="166" fontId="13" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="38" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="166" fontId="13" fillId="0" borderId="20" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="38" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="38" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="38" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="0" applyFont="1" applyProtection="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="0" borderId="0" xfId="0" applyFont="1" applyProtection="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="0" borderId="47" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="0" borderId="48" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="0" borderId="49" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="3" borderId="50" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="3" borderId="51" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="3" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="3" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="3" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="166" fontId="13" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="47" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="48" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="49" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="3" borderId="47" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="3" borderId="48" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="3" borderId="49" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="166" fontId="28" fillId="0" borderId="25" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="47" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="48" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="49" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
@@ -2062,10 +2417,6 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
     <xf numFmtId="0" fontId="26" fillId="0" borderId="47" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
@@ -2078,369 +2429,12 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="31" fillId="0" borderId="47" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="31" fillId="0" borderId="48" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="31" fillId="0" borderId="49" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
     <xf numFmtId="0" fontId="27" fillId="0" borderId="47" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
     </xf>
     <xf numFmtId="0" fontId="27" fillId="0" borderId="49" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="3" borderId="50" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="3" borderId="51" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="31" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="31" fillId="3" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="31" fillId="3" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="31" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="31" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="31" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="31" fillId="3" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="31" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="166" fontId="13" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="37" fillId="0" borderId="0" xfId="0" applyFont="1" applyProtection="1">
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="33" fillId="0" borderId="0" xfId="0" applyFont="1" applyProtection="1">
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="47" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="48" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="49" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="3" borderId="47" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="3" borderId="48" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="3" borderId="49" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="166" fontId="28" fillId="0" borderId="25" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="0" borderId="47" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="0" borderId="48" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="0" borderId="49" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="166" fontId="13" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="38" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="166" fontId="13" fillId="0" borderId="20" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="38" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="38" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="38" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="0" applyFont="1" applyProtection="1">
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="36" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="49" fontId="6" fillId="0" borderId="9" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="49" fontId="6" fillId="0" borderId="22" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="169" fontId="13" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="166" fontId="12" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="2" fontId="7" fillId="0" borderId="58" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="7" fillId="0" borderId="9" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="7" fillId="0" borderId="59" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="7" fillId="0" borderId="45" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="11" fillId="0" borderId="60" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="166" fontId="11" fillId="0" borderId="61" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="166" fontId="39" fillId="0" borderId="27" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="166" fontId="39" fillId="0" borderId="61" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="166" fontId="6" fillId="0" borderId="2" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="166" fontId="6" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="166" fontId="6" fillId="0" borderId="16" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="166" fontId="6" fillId="0" borderId="4" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="166" fontId="6" fillId="0" borderId="5" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="166" fontId="6" fillId="0" borderId="8" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="174" fontId="7" fillId="0" borderId="58" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="174" fontId="7" fillId="0" borderId="9" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="166" fontId="6" fillId="0" borderId="39" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="166" fontId="6" fillId="0" borderId="40" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="166" fontId="6" fillId="0" borderId="44" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="166" fontId="3" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="166" fontId="6" fillId="0" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="166" fontId="6" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="166" fontId="6" fillId="0" borderId="30" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="166" fontId="6" fillId="0" borderId="32" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="166" fontId="6" fillId="0" borderId="33" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="166" fontId="6" fillId="0" borderId="34" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="166" fontId="6" fillId="0" borderId="29" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="166" fontId="6" fillId="0" borderId="28" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="166" fontId="6" fillId="0" borderId="31" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="166" fontId="6" fillId="0" borderId="32" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="166" fontId="6" fillId="0" borderId="29" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="166" fontId="7" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="49" fontId="8" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="166" fontId="9" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="1" fontId="11" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
   </cellXfs>
@@ -2701,9 +2695,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2007 - 2010">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -2741,9 +2735,9 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2007 - 2010">
       <a:majorFont>
-        <a:latin typeface="Cambria" panose="020F0302020204030204"/>
+        <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -2776,26 +2770,9 @@
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
-        <a:font script="Armn" typeface="Arial"/>
-        <a:font script="Bugi" typeface="Leelawadee UI"/>
-        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
-        <a:font script="Java" typeface="Javanese Text"/>
-        <a:font script="Lisu" typeface="Segoe UI"/>
-        <a:font script="Mymr" typeface="Myanmar Text"/>
-        <a:font script="Nkoo" typeface="Ebrima"/>
-        <a:font script="Olck" typeface="Nirmala UI"/>
-        <a:font script="Osma" typeface="Ebrima"/>
-        <a:font script="Phag" typeface="Phagspa"/>
-        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
-        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
-        <a:font script="Syre" typeface="Estrangelo Edessa"/>
-        <a:font script="Sora" typeface="Nirmala UI"/>
-        <a:font script="Tale" typeface="Microsoft Tai Le"/>
-        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
-        <a:font script="Tfng" typeface="Ebrima"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
+        <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -2828,26 +2805,9 @@
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
-        <a:font script="Armn" typeface="Arial"/>
-        <a:font script="Bugi" typeface="Leelawadee UI"/>
-        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
-        <a:font script="Java" typeface="Javanese Text"/>
-        <a:font script="Lisu" typeface="Segoe UI"/>
-        <a:font script="Mymr" typeface="Myanmar Text"/>
-        <a:font script="Nkoo" typeface="Ebrima"/>
-        <a:font script="Olck" typeface="Nirmala UI"/>
-        <a:font script="Osma" typeface="Ebrima"/>
-        <a:font script="Phag" typeface="Phagspa"/>
-        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
-        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
-        <a:font script="Syre" typeface="Estrangelo Edessa"/>
-        <a:font script="Sora" typeface="Nirmala UI"/>
-        <a:font script="Tale" typeface="Microsoft Tai Le"/>
-        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
-        <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2007 - 2010">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -3023,70 +2983,70 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BB524E58-DEC5-4CFF-AD7C-0D1451F04347}">
   <sheetPr codeName="Sheet2"/>
   <dimension ref="A1:R148"/>
-  <sheetFormatPr defaultColWidth="9.1796875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="12.1796875" style="8" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="8.453125" style="8" customWidth="1"/>
-    <col min="3" max="3" width="8.54296875" style="8" customWidth="1"/>
-    <col min="4" max="4" width="9.1796875" style="8"/>
-    <col min="5" max="5" width="8.54296875" style="8" customWidth="1"/>
+    <col min="1" max="1" width="12.140625" style="8" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="8.42578125" style="8" customWidth="1"/>
+    <col min="3" max="3" width="8.5703125" style="8" customWidth="1"/>
+    <col min="4" max="4" width="9.140625" style="8"/>
+    <col min="5" max="5" width="8.5703125" style="8" customWidth="1"/>
     <col min="6" max="6" width="12" style="8" customWidth="1"/>
-    <col min="7" max="8" width="9.26953125" style="8" customWidth="1"/>
+    <col min="7" max="8" width="9.28515625" style="8" customWidth="1"/>
     <col min="9" max="9" width="10" style="8" customWidth="1"/>
-    <col min="10" max="11" width="9.26953125" style="8" customWidth="1"/>
-    <col min="12" max="12" width="15.26953125" style="8" customWidth="1"/>
-    <col min="13" max="13" width="13.1796875" style="8" customWidth="1"/>
-    <col min="14" max="15" width="7.453125" style="8" customWidth="1"/>
-    <col min="16" max="16" width="28.26953125" style="8" customWidth="1"/>
-    <col min="17" max="17" width="30.54296875" style="8" customWidth="1"/>
-    <col min="18" max="18" width="31.81640625" style="8" customWidth="1"/>
-    <col min="19" max="16384" width="9.1796875" style="8"/>
+    <col min="10" max="11" width="9.28515625" style="8" customWidth="1"/>
+    <col min="12" max="12" width="15.28515625" style="8" customWidth="1"/>
+    <col min="13" max="13" width="13.140625" style="8" customWidth="1"/>
+    <col min="14" max="15" width="7.42578125" style="8" customWidth="1"/>
+    <col min="16" max="16" width="28.28515625" style="8" customWidth="1"/>
+    <col min="17" max="17" width="30.5703125" style="8" customWidth="1"/>
+    <col min="18" max="18" width="31.85546875" style="8" customWidth="1"/>
+    <col min="19" max="16384" width="9.140625" style="8"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:18" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A1" s="242" t="s">
+    <row r="1" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A1" s="164" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="242"/>
-      <c r="C1" s="242"/>
-      <c r="D1" s="242"/>
-      <c r="E1" s="242"/>
-      <c r="F1" s="242"/>
-      <c r="G1" s="242"/>
-      <c r="H1" s="242"/>
-      <c r="I1" s="242"/>
-      <c r="J1" s="242"/>
-      <c r="K1" s="242"/>
-      <c r="L1" s="242"/>
+      <c r="B1" s="164"/>
+      <c r="C1" s="164"/>
+      <c r="D1" s="164"/>
+      <c r="E1" s="164"/>
+      <c r="F1" s="164"/>
+      <c r="G1" s="164"/>
+      <c r="H1" s="164"/>
+      <c r="I1" s="164"/>
+      <c r="J1" s="164"/>
+      <c r="K1" s="164"/>
+      <c r="L1" s="164"/>
       <c r="M1" s="9"/>
       <c r="N1" s="9"/>
       <c r="O1" s="9"/>
       <c r="P1" s="9"/>
       <c r="Q1" s="9"/>
     </row>
-    <row r="2" spans="1:18" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A2" s="242" t="s">
+    <row r="2" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A2" s="164" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="242"/>
-      <c r="C2" s="242"/>
-      <c r="D2" s="242"/>
-      <c r="E2" s="242"/>
-      <c r="F2" s="242"/>
-      <c r="G2" s="242"/>
-      <c r="H2" s="242"/>
-      <c r="I2" s="242"/>
-      <c r="J2" s="242"/>
-      <c r="K2" s="242"/>
-      <c r="L2" s="242"/>
-      <c r="M2" s="231"/>
-      <c r="N2" s="231"/>
-      <c r="O2" s="231"/>
-      <c r="P2" s="231"/>
-      <c r="Q2" s="231"/>
-      <c r="R2" s="231"/>
-    </row>
-    <row r="3" spans="1:18" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="B2" s="164"/>
+      <c r="C2" s="164"/>
+      <c r="D2" s="164"/>
+      <c r="E2" s="164"/>
+      <c r="F2" s="164"/>
+      <c r="G2" s="164"/>
+      <c r="H2" s="164"/>
+      <c r="I2" s="164"/>
+      <c r="J2" s="164"/>
+      <c r="K2" s="164"/>
+      <c r="L2" s="164"/>
+      <c r="M2" s="151"/>
+      <c r="N2" s="151"/>
+      <c r="O2" s="151"/>
+      <c r="P2" s="151"/>
+      <c r="Q2" s="151"/>
+      <c r="R2" s="151"/>
+    </row>
+    <row r="3" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A3" s="10"/>
       <c r="B3" s="11"/>
       <c r="C3" s="11"/>
@@ -3104,39 +3064,39 @@
       <c r="Q3" s="9"/>
       <c r="R3" s="9"/>
     </row>
-    <row r="4" spans="1:18" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A4" s="254" t="s">
+    <row r="4" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A4" s="177" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="254"/>
-      <c r="C4" s="254"/>
-      <c r="D4" s="254"/>
-      <c r="E4" s="254"/>
-      <c r="F4" s="254"/>
-      <c r="G4" s="254"/>
-      <c r="H4" s="254"/>
-      <c r="I4" s="254"/>
-      <c r="J4" s="254"/>
-      <c r="K4" s="254"/>
-      <c r="L4" s="254"/>
+      <c r="B4" s="177"/>
+      <c r="C4" s="177"/>
+      <c r="D4" s="177"/>
+      <c r="E4" s="177"/>
+      <c r="F4" s="177"/>
+      <c r="G4" s="177"/>
+      <c r="H4" s="177"/>
+      <c r="I4" s="177"/>
+      <c r="J4" s="177"/>
+      <c r="K4" s="177"/>
+      <c r="L4" s="177"/>
       <c r="O4" s="9"/>
       <c r="P4" s="9"/>
       <c r="Q4" s="9"/>
       <c r="R4" s="9"/>
     </row>
-    <row r="5" spans="1:18" ht="17.5" x14ac:dyDescent="0.35">
-      <c r="A5" s="255"/>
-      <c r="B5" s="255"/>
-      <c r="C5" s="255"/>
-      <c r="D5" s="255"/>
-      <c r="E5" s="255"/>
-      <c r="F5" s="255"/>
-      <c r="G5" s="255"/>
-      <c r="H5" s="255"/>
-      <c r="I5" s="255"/>
-      <c r="J5" s="255"/>
-      <c r="K5" s="255"/>
-      <c r="L5" s="255"/>
+    <row r="5" spans="1:18" ht="18" x14ac:dyDescent="0.25">
+      <c r="A5" s="178"/>
+      <c r="B5" s="178"/>
+      <c r="C5" s="178"/>
+      <c r="D5" s="178"/>
+      <c r="E5" s="178"/>
+      <c r="F5" s="178"/>
+      <c r="G5" s="178"/>
+      <c r="H5" s="178"/>
+      <c r="I5" s="178"/>
+      <c r="J5" s="178"/>
+      <c r="K5" s="178"/>
+      <c r="L5" s="178"/>
       <c r="O5" s="9"/>
       <c r="P5" s="9"/>
       <c r="Q5" s="9"/>
@@ -3144,27 +3104,27 @@
         <v>58</v>
       </c>
     </row>
-    <row r="6" spans="1:18" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A6" s="256" t="s">
+    <row r="6" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A6" s="179" t="s">
         <v>3</v>
       </c>
-      <c r="B6" s="256"/>
-      <c r="C6" s="256"/>
-      <c r="D6" s="256"/>
-      <c r="E6" s="256"/>
-      <c r="F6" s="256"/>
-      <c r="G6" s="256"/>
-      <c r="H6" s="256"/>
-      <c r="I6" s="256"/>
-      <c r="J6" s="256"/>
-      <c r="K6" s="256"/>
-      <c r="L6" s="256"/>
+      <c r="B6" s="179"/>
+      <c r="C6" s="179"/>
+      <c r="D6" s="179"/>
+      <c r="E6" s="179"/>
+      <c r="F6" s="179"/>
+      <c r="G6" s="179"/>
+      <c r="H6" s="179"/>
+      <c r="I6" s="179"/>
+      <c r="J6" s="179"/>
+      <c r="K6" s="179"/>
+      <c r="L6" s="179"/>
       <c r="O6" s="16"/>
       <c r="P6" s="9"/>
       <c r="Q6" s="9"/>
       <c r="R6" s="9"/>
     </row>
-    <row r="7" spans="1:18" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A7" s="17"/>
       <c r="B7" s="18"/>
       <c r="C7" s="18"/>
@@ -3184,7 +3144,7 @@
       <c r="Q7" s="9"/>
       <c r="R7" s="9"/>
     </row>
-    <row r="8" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="19" t="s">
         <v>4</v>
       </c>
@@ -3206,16 +3166,16 @@
       </c>
       <c r="L8" s="136"/>
     </row>
-    <row r="9" spans="1:18" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A9" s="19" t="s">
         <v>86</v>
       </c>
       <c r="B9" s="20" t="s">
         <v>5</v>
       </c>
-      <c r="C9" s="257"/>
-      <c r="D9" s="257"/>
-      <c r="E9" s="257"/>
+      <c r="C9" s="180"/>
+      <c r="D9" s="180"/>
+      <c r="E9" s="180"/>
       <c r="F9" s="22"/>
       <c r="G9" s="22"/>
       <c r="H9" s="19" t="s">
@@ -3228,7 +3188,7 @@
       </c>
       <c r="L9" s="137"/>
       <c r="M9" s="144" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="N9" s="9"/>
       <c r="O9" s="24"/>
@@ -3237,7 +3197,7 @@
         <v xml:space="preserve">:   </v>
       </c>
     </row>
-    <row r="10" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="19" t="s">
         <v>8</v>
       </c>
@@ -3261,7 +3221,7 @@
         <v>10</v>
       </c>
       <c r="M10" s="144" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="N10" s="9"/>
       <c r="O10" s="24"/>
@@ -3270,7 +3230,7 @@
         <v xml:space="preserve">:   </v>
       </c>
     </row>
-    <row r="11" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="19" t="s">
         <v>11</v>
       </c>
@@ -3292,7 +3252,7 @@
       </c>
       <c r="L11" s="138"/>
       <c r="M11" s="144" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="N11" s="9"/>
       <c r="O11" s="24"/>
@@ -3301,7 +3261,7 @@
         <v xml:space="preserve">:   </v>
       </c>
     </row>
-    <row r="12" spans="1:18" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A12" s="19" t="s">
         <v>13</v>
       </c>
@@ -3323,7 +3283,7 @@
       </c>
       <c r="L12" s="138"/>
       <c r="M12" s="145" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="N12" s="16"/>
       <c r="O12" s="24"/>
@@ -3332,7 +3292,7 @@
         <v xml:space="preserve">:   </v>
       </c>
     </row>
-    <row r="13" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A13" s="19"/>
       <c r="B13" s="21"/>
       <c r="C13" s="26"/>
@@ -3346,7 +3306,7 @@
       <c r="K13" s="20"/>
       <c r="L13" s="26"/>
     </row>
-    <row r="14" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="14" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A14" s="17"/>
       <c r="B14" s="18"/>
       <c r="C14" s="18"/>
@@ -3360,71 +3320,71 @@
       <c r="K14" s="12"/>
       <c r="L14" s="26"/>
     </row>
-    <row r="15" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="28" t="s">
         <v>15</v>
       </c>
-      <c r="B15" s="243" t="s">
+      <c r="B15" s="165" t="s">
         <v>16</v>
       </c>
-      <c r="C15" s="243"/>
-      <c r="D15" s="245" t="s">
+      <c r="C15" s="165"/>
+      <c r="D15" s="167" t="s">
         <v>17</v>
       </c>
-      <c r="E15" s="246"/>
-      <c r="F15" s="246" t="s">
+      <c r="E15" s="168"/>
+      <c r="F15" s="168" t="s">
         <v>18</v>
       </c>
-      <c r="G15" s="251" t="s">
+      <c r="G15" s="173" t="s">
         <v>19</v>
       </c>
-      <c r="H15" s="251"/>
-      <c r="I15" s="251"/>
-      <c r="J15" s="251"/>
-      <c r="K15" s="252"/>
-      <c r="L15" s="232" t="s">
+      <c r="H15" s="173"/>
+      <c r="I15" s="173"/>
+      <c r="J15" s="173"/>
+      <c r="K15" s="174"/>
+      <c r="L15" s="154" t="s">
         <v>20</v>
       </c>
-      <c r="M15" s="235" t="s">
+      <c r="M15" s="157" t="s">
         <v>59</v>
       </c>
-      <c r="N15" s="238" t="s">
+      <c r="N15" s="160" t="s">
         <v>60</v>
       </c>
-      <c r="O15" s="239"/>
-      <c r="P15" s="235" t="s">
+      <c r="O15" s="161"/>
+      <c r="P15" s="157" t="s">
         <v>61</v>
       </c>
-      <c r="Q15" s="258" t="s">
+      <c r="Q15" s="181" t="s">
         <v>62</v>
       </c>
-      <c r="R15" s="235" t="s">
+      <c r="R15" s="157" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="16" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="16" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A16" s="29" t="s">
         <v>21</v>
       </c>
-      <c r="B16" s="244"/>
-      <c r="C16" s="244"/>
-      <c r="D16" s="247"/>
-      <c r="E16" s="248"/>
-      <c r="F16" s="249"/>
-      <c r="G16" s="224"/>
-      <c r="H16" s="224"/>
-      <c r="I16" s="224"/>
-      <c r="J16" s="224"/>
-      <c r="K16" s="253"/>
-      <c r="L16" s="233"/>
-      <c r="M16" s="236"/>
-      <c r="N16" s="240"/>
-      <c r="O16" s="241"/>
-      <c r="P16" s="236"/>
-      <c r="Q16" s="259"/>
-      <c r="R16" s="236"/>
-    </row>
-    <row r="17" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="B16" s="166"/>
+      <c r="C16" s="166"/>
+      <c r="D16" s="169"/>
+      <c r="E16" s="170"/>
+      <c r="F16" s="171"/>
+      <c r="G16" s="175"/>
+      <c r="H16" s="175"/>
+      <c r="I16" s="175"/>
+      <c r="J16" s="175"/>
+      <c r="K16" s="176"/>
+      <c r="L16" s="155"/>
+      <c r="M16" s="158"/>
+      <c r="N16" s="162"/>
+      <c r="O16" s="163"/>
+      <c r="P16" s="158"/>
+      <c r="Q16" s="182"/>
+      <c r="R16" s="158"/>
+    </row>
+    <row r="17" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A17" s="30" t="s">
         <v>22</v>
       </c>
@@ -3440,7 +3400,7 @@
       <c r="E17" s="34" t="s">
         <v>24</v>
       </c>
-      <c r="F17" s="250"/>
+      <c r="F17" s="172"/>
       <c r="G17" s="35" t="s">
         <v>25</v>
       </c>
@@ -3456,1011 +3416,1007 @@
       <c r="K17" s="37">
         <v>2</v>
       </c>
-      <c r="L17" s="234"/>
-      <c r="M17" s="237"/>
+      <c r="L17" s="156"/>
+      <c r="M17" s="159"/>
       <c r="N17" s="38" t="s">
         <v>23</v>
       </c>
       <c r="O17" s="38" t="s">
         <v>24</v>
       </c>
-      <c r="P17" s="237"/>
-      <c r="Q17" s="260"/>
-      <c r="R17" s="237"/>
-    </row>
-    <row r="18" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A18" s="223" t="s">
-        <v>109</v>
-      </c>
-      <c r="B18" s="224"/>
-      <c r="C18" s="224"/>
-      <c r="D18" s="224"/>
-      <c r="E18" s="225"/>
-      <c r="F18" s="229"/>
-      <c r="G18" s="212"/>
-      <c r="H18" s="212">
+      <c r="P17" s="159"/>
+      <c r="Q17" s="183"/>
+      <c r="R17" s="159"/>
+    </row>
+    <row r="18" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A18" s="195" t="s">
+        <v>107</v>
+      </c>
+      <c r="B18" s="175"/>
+      <c r="C18" s="175"/>
+      <c r="D18" s="175"/>
+      <c r="E18" s="196"/>
+      <c r="F18" s="200"/>
+      <c r="G18" s="152"/>
+      <c r="H18" s="152">
         <f>F18</f>
         <v>0</v>
       </c>
-      <c r="I18" s="212"/>
-      <c r="J18" s="212"/>
-      <c r="K18" s="214"/>
-      <c r="L18" s="216" t="s">
-        <v>110</v>
+      <c r="I18" s="152"/>
+      <c r="J18" s="152"/>
+      <c r="K18" s="186"/>
+      <c r="L18" s="188" t="s">
+        <v>108</v>
       </c>
       <c r="M18" s="147" t="str">
         <f>IF(ISBLANK(A20),"",A20)</f>
         <v/>
       </c>
-      <c r="N18" s="153" t="str">
+      <c r="N18" s="208" t="str">
         <f>IF(ISBLANK(D20),"",D20)</f>
         <v/>
       </c>
-      <c r="O18" s="154"/>
-      <c r="P18" s="218" t="s">
-        <v>88</v>
-      </c>
-      <c r="Q18" s="207"/>
+      <c r="O18" s="209"/>
+      <c r="P18" s="190"/>
+      <c r="Q18" s="211"/>
       <c r="R18" s="149"/>
     </row>
-    <row r="19" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A19" s="226"/>
-      <c r="B19" s="227"/>
-      <c r="C19" s="227"/>
-      <c r="D19" s="227"/>
-      <c r="E19" s="228"/>
-      <c r="F19" s="230"/>
-      <c r="G19" s="213"/>
-      <c r="H19" s="213"/>
-      <c r="I19" s="213"/>
-      <c r="J19" s="213"/>
-      <c r="K19" s="215"/>
-      <c r="L19" s="217"/>
+    <row r="19" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A19" s="197"/>
+      <c r="B19" s="198"/>
+      <c r="C19" s="198"/>
+      <c r="D19" s="198"/>
+      <c r="E19" s="199"/>
+      <c r="F19" s="201"/>
+      <c r="G19" s="153"/>
+      <c r="H19" s="153"/>
+      <c r="I19" s="153"/>
+      <c r="J19" s="153"/>
+      <c r="K19" s="187"/>
+      <c r="L19" s="189"/>
       <c r="M19" s="148" t="str">
         <f>A21</f>
         <v/>
       </c>
-      <c r="N19" s="151" t="str">
+      <c r="N19" s="206" t="str">
         <f>IF(ISBLANK(D21),"",D21)</f>
         <v/>
       </c>
-      <c r="O19" s="152"/>
-      <c r="P19" s="219"/>
-      <c r="Q19" s="208"/>
+      <c r="O19" s="207"/>
+      <c r="P19" s="191"/>
+      <c r="Q19" s="212"/>
       <c r="R19" s="150"/>
     </row>
-    <row r="20" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="142"/>
-      <c r="B20" s="206"/>
-      <c r="C20" s="206"/>
-      <c r="D20" s="155"/>
-      <c r="E20" s="156"/>
+      <c r="B20" s="185"/>
+      <c r="C20" s="185"/>
+      <c r="D20" s="204"/>
+      <c r="E20" s="205"/>
       <c r="F20" s="139"/>
       <c r="G20" s="129"/>
       <c r="H20" s="129"/>
       <c r="I20" s="129"/>
       <c r="J20" s="129"/>
       <c r="K20" s="129"/>
-      <c r="L20" s="221" t="s">
-        <v>87</v>
-      </c>
+      <c r="L20" s="193"/>
       <c r="M20" s="147" t="str">
         <f>IF(ISBLANK(A22),"",A22)</f>
         <v/>
       </c>
-      <c r="N20" s="153" t="str">
+      <c r="N20" s="208" t="str">
         <f t="shared" ref="N20:N53" si="0">IF(ISBLANK(D22),"",D22)</f>
         <v/>
       </c>
-      <c r="O20" s="154"/>
-      <c r="P20" s="219"/>
-      <c r="Q20" s="208"/>
+      <c r="O20" s="209"/>
+      <c r="P20" s="191"/>
+      <c r="Q20" s="212"/>
       <c r="R20" s="149"/>
     </row>
-    <row r="21" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="1" t="str">
         <f t="shared" ref="A21" si="1">IF(A20="","",UPPER(TEXT(A20,"[$-043E]DDDD")))</f>
         <v/>
       </c>
-      <c r="B21" s="206"/>
-      <c r="C21" s="206"/>
-      <c r="D21" s="157"/>
-      <c r="E21" s="158"/>
+      <c r="B21" s="185"/>
+      <c r="C21" s="185"/>
+      <c r="D21" s="202"/>
+      <c r="E21" s="203"/>
       <c r="F21" s="141"/>
       <c r="G21" s="127"/>
       <c r="H21" s="127"/>
       <c r="I21" s="127"/>
       <c r="J21" s="127"/>
       <c r="K21" s="128"/>
-      <c r="L21" s="221"/>
+      <c r="L21" s="193"/>
       <c r="M21" s="148" t="str">
         <f>A23</f>
         <v/>
       </c>
-      <c r="N21" s="151" t="str">
+      <c r="N21" s="206" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
-      <c r="O21" s="152"/>
-      <c r="P21" s="219"/>
-      <c r="Q21" s="208"/>
+      <c r="O21" s="207"/>
+      <c r="P21" s="191"/>
+      <c r="Q21" s="212"/>
       <c r="R21" s="150"/>
     </row>
-    <row r="22" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="134"/>
-      <c r="B22" s="205"/>
-      <c r="C22" s="205"/>
-      <c r="D22" s="155"/>
-      <c r="E22" s="156"/>
+      <c r="B22" s="184"/>
+      <c r="C22" s="184"/>
+      <c r="D22" s="204"/>
+      <c r="E22" s="205"/>
       <c r="F22" s="139"/>
       <c r="G22" s="129"/>
       <c r="H22" s="129"/>
       <c r="I22" s="129"/>
       <c r="J22" s="129"/>
       <c r="K22" s="129"/>
-      <c r="L22" s="221"/>
+      <c r="L22" s="193"/>
       <c r="M22" s="147" t="str">
         <f t="shared" ref="M22" si="2">IF(ISBLANK(A24),"",A24)</f>
         <v/>
       </c>
-      <c r="N22" s="153" t="str">
+      <c r="N22" s="208" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
-      <c r="O22" s="154"/>
-      <c r="P22" s="219"/>
-      <c r="Q22" s="208"/>
+      <c r="O22" s="209"/>
+      <c r="P22" s="191"/>
+      <c r="Q22" s="212"/>
       <c r="R22" s="149"/>
     </row>
-    <row r="23" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="1" t="str">
         <f t="shared" ref="A23:A25" si="3">IF(A22="","",UPPER(TEXT(A22,"[$-043E]DDDD")))</f>
         <v/>
       </c>
-      <c r="B23" s="206"/>
-      <c r="C23" s="206"/>
-      <c r="D23" s="157"/>
-      <c r="E23" s="158"/>
+      <c r="B23" s="185"/>
+      <c r="C23" s="185"/>
+      <c r="D23" s="202"/>
+      <c r="E23" s="203"/>
       <c r="F23" s="141"/>
       <c r="G23" s="127"/>
       <c r="H23" s="127"/>
       <c r="I23" s="127"/>
       <c r="J23" s="127"/>
       <c r="K23" s="128"/>
-      <c r="L23" s="221"/>
+      <c r="L23" s="193"/>
       <c r="M23" s="148" t="str">
         <f t="shared" ref="M23" si="4">A25</f>
         <v/>
       </c>
-      <c r="N23" s="151" t="str">
+      <c r="N23" s="206" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
-      <c r="O23" s="152"/>
-      <c r="P23" s="219"/>
-      <c r="Q23" s="208"/>
+      <c r="O23" s="207"/>
+      <c r="P23" s="191"/>
+      <c r="Q23" s="212"/>
       <c r="R23" s="150"/>
     </row>
-    <row r="24" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="134"/>
-      <c r="B24" s="205"/>
-      <c r="C24" s="205"/>
-      <c r="D24" s="155"/>
-      <c r="E24" s="156"/>
+      <c r="B24" s="184"/>
+      <c r="C24" s="184"/>
+      <c r="D24" s="204"/>
+      <c r="E24" s="205"/>
       <c r="F24" s="139"/>
       <c r="G24" s="129"/>
       <c r="H24" s="129"/>
       <c r="I24" s="129"/>
       <c r="J24" s="129"/>
       <c r="K24" s="129"/>
-      <c r="L24" s="221"/>
+      <c r="L24" s="193"/>
       <c r="M24" s="147" t="str">
         <f t="shared" ref="M24" si="5">IF(ISBLANK(A26),"",A26)</f>
         <v/>
       </c>
-      <c r="N24" s="153" t="str">
+      <c r="N24" s="208" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
-      <c r="O24" s="154"/>
-      <c r="P24" s="219"/>
-      <c r="Q24" s="208"/>
+      <c r="O24" s="209"/>
+      <c r="P24" s="191"/>
+      <c r="Q24" s="212"/>
       <c r="R24" s="149"/>
     </row>
-    <row r="25" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="1" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
-      <c r="B25" s="206"/>
-      <c r="C25" s="206"/>
-      <c r="D25" s="157"/>
-      <c r="E25" s="158"/>
+      <c r="B25" s="185"/>
+      <c r="C25" s="185"/>
+      <c r="D25" s="202"/>
+      <c r="E25" s="203"/>
       <c r="F25" s="141"/>
       <c r="G25" s="127"/>
       <c r="H25" s="127"/>
       <c r="I25" s="127"/>
       <c r="J25" s="127"/>
       <c r="K25" s="128"/>
-      <c r="L25" s="221"/>
+      <c r="L25" s="193"/>
       <c r="M25" s="148" t="str">
         <f t="shared" ref="M25" si="6">A27</f>
         <v/>
       </c>
-      <c r="N25" s="151" t="str">
+      <c r="N25" s="206" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
-      <c r="O25" s="152"/>
-      <c r="P25" s="219"/>
-      <c r="Q25" s="208"/>
+      <c r="O25" s="207"/>
+      <c r="P25" s="191"/>
+      <c r="Q25" s="212"/>
       <c r="R25" s="150"/>
     </row>
-    <row r="26" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="134"/>
-      <c r="B26" s="205"/>
-      <c r="C26" s="205"/>
-      <c r="D26" s="155"/>
-      <c r="E26" s="156"/>
+      <c r="B26" s="184"/>
+      <c r="C26" s="184"/>
+      <c r="D26" s="204"/>
+      <c r="E26" s="205"/>
       <c r="F26" s="139"/>
       <c r="G26" s="129"/>
       <c r="H26" s="129"/>
       <c r="I26" s="129"/>
       <c r="J26" s="129"/>
       <c r="K26" s="129"/>
-      <c r="L26" s="221"/>
+      <c r="L26" s="193"/>
       <c r="M26" s="147" t="str">
         <f t="shared" ref="M26" si="7">IF(ISBLANK(A28),"",A28)</f>
         <v/>
       </c>
-      <c r="N26" s="153" t="str">
+      <c r="N26" s="208" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
-      <c r="O26" s="154"/>
-      <c r="P26" s="219"/>
-      <c r="Q26" s="208"/>
+      <c r="O26" s="209"/>
+      <c r="P26" s="191"/>
+      <c r="Q26" s="212"/>
       <c r="R26" s="149"/>
     </row>
-    <row r="27" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="1" t="str">
         <f t="shared" ref="A27" si="8">IF(A26="","",UPPER(TEXT(A26,"[$-043E]DDDD")))</f>
         <v/>
       </c>
-      <c r="B27" s="206"/>
-      <c r="C27" s="206"/>
-      <c r="D27" s="157"/>
-      <c r="E27" s="158"/>
+      <c r="B27" s="185"/>
+      <c r="C27" s="185"/>
+      <c r="D27" s="202"/>
+      <c r="E27" s="203"/>
       <c r="F27" s="141"/>
       <c r="G27" s="127"/>
       <c r="H27" s="127"/>
       <c r="I27" s="127"/>
       <c r="J27" s="127"/>
       <c r="K27" s="128"/>
-      <c r="L27" s="221"/>
+      <c r="L27" s="193"/>
       <c r="M27" s="148" t="str">
         <f t="shared" ref="M27" si="9">A29</f>
         <v/>
       </c>
-      <c r="N27" s="151" t="str">
+      <c r="N27" s="206" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
-      <c r="O27" s="152"/>
-      <c r="P27" s="219"/>
-      <c r="Q27" s="208"/>
+      <c r="O27" s="207"/>
+      <c r="P27" s="191"/>
+      <c r="Q27" s="212"/>
       <c r="R27" s="150"/>
     </row>
-    <row r="28" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="135"/>
-      <c r="B28" s="205"/>
-      <c r="C28" s="205"/>
-      <c r="D28" s="155"/>
-      <c r="E28" s="156"/>
+      <c r="B28" s="184"/>
+      <c r="C28" s="184"/>
+      <c r="D28" s="204"/>
+      <c r="E28" s="205"/>
       <c r="F28" s="139"/>
       <c r="G28" s="129"/>
       <c r="H28" s="129"/>
       <c r="I28" s="129"/>
       <c r="J28" s="129"/>
       <c r="K28" s="129"/>
-      <c r="L28" s="221"/>
+      <c r="L28" s="193"/>
       <c r="M28" s="147" t="str">
         <f t="shared" ref="M28" si="10">IF(ISBLANK(A30),"",A30)</f>
         <v/>
       </c>
-      <c r="N28" s="153" t="str">
+      <c r="N28" s="208" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
-      <c r="O28" s="154"/>
-      <c r="P28" s="219"/>
-      <c r="Q28" s="208"/>
+      <c r="O28" s="209"/>
+      <c r="P28" s="191"/>
+      <c r="Q28" s="212"/>
       <c r="R28" s="149"/>
     </row>
-    <row r="29" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="6" t="str">
         <f t="shared" ref="A29" si="11">IF(A28="","",UPPER(TEXT(A28,"[$-043E]DDDD")))</f>
         <v/>
       </c>
-      <c r="B29" s="206"/>
-      <c r="C29" s="206"/>
-      <c r="D29" s="157"/>
-      <c r="E29" s="158"/>
+      <c r="B29" s="185"/>
+      <c r="C29" s="185"/>
+      <c r="D29" s="202"/>
+      <c r="E29" s="203"/>
       <c r="F29" s="141"/>
       <c r="G29" s="127"/>
       <c r="H29" s="127"/>
       <c r="I29" s="127"/>
       <c r="J29" s="129"/>
       <c r="K29" s="128"/>
-      <c r="L29" s="221"/>
+      <c r="L29" s="193"/>
       <c r="M29" s="148" t="str">
         <f t="shared" ref="M29" si="12">A31</f>
         <v/>
       </c>
-      <c r="N29" s="151" t="str">
+      <c r="N29" s="206" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
-      <c r="O29" s="152"/>
-      <c r="P29" s="219"/>
-      <c r="Q29" s="208"/>
+      <c r="O29" s="207"/>
+      <c r="P29" s="191"/>
+      <c r="Q29" s="212"/>
       <c r="R29" s="150"/>
     </row>
-    <row r="30" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30" s="134"/>
-      <c r="B30" s="205"/>
-      <c r="C30" s="205"/>
-      <c r="D30" s="155"/>
-      <c r="E30" s="156"/>
+      <c r="B30" s="184"/>
+      <c r="C30" s="184"/>
+      <c r="D30" s="204"/>
+      <c r="E30" s="205"/>
       <c r="F30" s="139"/>
       <c r="G30" s="129"/>
       <c r="H30" s="129"/>
       <c r="I30" s="140"/>
       <c r="J30" s="143"/>
       <c r="K30" s="139"/>
-      <c r="L30" s="221"/>
+      <c r="L30" s="193"/>
       <c r="M30" s="147" t="str">
         <f t="shared" ref="M30" si="13">IF(ISBLANK(A32),"",A32)</f>
         <v/>
       </c>
-      <c r="N30" s="153" t="str">
+      <c r="N30" s="208" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
-      <c r="O30" s="154"/>
-      <c r="P30" s="219"/>
-      <c r="Q30" s="208"/>
+      <c r="O30" s="209"/>
+      <c r="P30" s="191"/>
+      <c r="Q30" s="212"/>
       <c r="R30" s="149"/>
     </row>
-    <row r="31" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" s="1" t="str">
         <f t="shared" ref="A31" si="14">IF(A30="","",UPPER(TEXT(A30,"[$-043E]DDDD")))</f>
         <v/>
       </c>
-      <c r="B31" s="206"/>
-      <c r="C31" s="206"/>
-      <c r="D31" s="157"/>
-      <c r="E31" s="158"/>
+      <c r="B31" s="185"/>
+      <c r="C31" s="185"/>
+      <c r="D31" s="202"/>
+      <c r="E31" s="203"/>
       <c r="F31" s="141"/>
       <c r="G31" s="127"/>
       <c r="H31" s="127"/>
       <c r="I31" s="127"/>
       <c r="J31" s="127"/>
       <c r="K31" s="128"/>
-      <c r="L31" s="221"/>
+      <c r="L31" s="193"/>
       <c r="M31" s="148" t="str">
         <f t="shared" ref="M31" si="15">A33</f>
         <v/>
       </c>
-      <c r="N31" s="151" t="str">
+      <c r="N31" s="206" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
-      <c r="O31" s="152"/>
-      <c r="P31" s="219"/>
-      <c r="Q31" s="208"/>
+      <c r="O31" s="207"/>
+      <c r="P31" s="191"/>
+      <c r="Q31" s="212"/>
       <c r="R31" s="150"/>
     </row>
-    <row r="32" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A32" s="134"/>
-      <c r="B32" s="205"/>
-      <c r="C32" s="205"/>
-      <c r="D32" s="155"/>
-      <c r="E32" s="156"/>
+      <c r="B32" s="184"/>
+      <c r="C32" s="184"/>
+      <c r="D32" s="204"/>
+      <c r="E32" s="205"/>
       <c r="F32" s="139"/>
       <c r="G32" s="129"/>
       <c r="H32" s="129"/>
       <c r="I32" s="129"/>
       <c r="J32" s="129"/>
       <c r="K32" s="129"/>
-      <c r="L32" s="221"/>
+      <c r="L32" s="193"/>
       <c r="M32" s="147" t="str">
         <f t="shared" ref="M32" si="16">IF(ISBLANK(A34),"",A34)</f>
         <v/>
       </c>
-      <c r="N32" s="153" t="str">
+      <c r="N32" s="208" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
-      <c r="O32" s="154"/>
-      <c r="P32" s="219"/>
-      <c r="Q32" s="208"/>
+      <c r="O32" s="209"/>
+      <c r="P32" s="191"/>
+      <c r="Q32" s="212"/>
       <c r="R32" s="149"/>
     </row>
-    <row r="33" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A33" s="1" t="str">
         <f t="shared" ref="A33" si="17">IF(A32="","",UPPER(TEXT(A32,"[$-043E]DDDD")))</f>
         <v/>
       </c>
-      <c r="B33" s="206"/>
-      <c r="C33" s="206"/>
-      <c r="D33" s="157"/>
-      <c r="E33" s="158"/>
+      <c r="B33" s="185"/>
+      <c r="C33" s="185"/>
+      <c r="D33" s="202"/>
+      <c r="E33" s="203"/>
       <c r="F33" s="141"/>
       <c r="G33" s="127"/>
       <c r="H33" s="127"/>
       <c r="I33" s="127"/>
       <c r="J33" s="127"/>
       <c r="K33" s="128"/>
-      <c r="L33" s="221"/>
+      <c r="L33" s="193"/>
       <c r="M33" s="148" t="str">
         <f t="shared" ref="M33" si="18">A35</f>
         <v/>
       </c>
-      <c r="N33" s="151" t="str">
+      <c r="N33" s="206" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
-      <c r="O33" s="152"/>
-      <c r="P33" s="219"/>
-      <c r="Q33" s="208"/>
+      <c r="O33" s="207"/>
+      <c r="P33" s="191"/>
+      <c r="Q33" s="212"/>
       <c r="R33" s="150"/>
     </row>
-    <row r="34" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A34" s="134"/>
-      <c r="B34" s="205"/>
-      <c r="C34" s="205"/>
-      <c r="D34" s="155"/>
-      <c r="E34" s="156"/>
+      <c r="B34" s="184"/>
+      <c r="C34" s="184"/>
+      <c r="D34" s="204"/>
+      <c r="E34" s="205"/>
       <c r="F34" s="139"/>
       <c r="G34" s="129"/>
       <c r="H34" s="129"/>
       <c r="I34" s="129"/>
       <c r="J34" s="129"/>
       <c r="K34" s="129"/>
-      <c r="L34" s="221"/>
+      <c r="L34" s="193"/>
       <c r="M34" s="147" t="str">
         <f t="shared" ref="M34" si="19">IF(ISBLANK(A36),"",A36)</f>
         <v/>
       </c>
-      <c r="N34" s="153" t="str">
+      <c r="N34" s="208" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
-      <c r="O34" s="154"/>
-      <c r="P34" s="219"/>
-      <c r="Q34" s="208"/>
+      <c r="O34" s="209"/>
+      <c r="P34" s="191"/>
+      <c r="Q34" s="212"/>
       <c r="R34" s="149"/>
     </row>
-    <row r="35" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A35" s="1" t="str">
         <f t="shared" ref="A35" si="20">IF(A34="","",UPPER(TEXT(A34,"[$-043E]DDDD")))</f>
         <v/>
       </c>
-      <c r="B35" s="206"/>
-      <c r="C35" s="206"/>
-      <c r="D35" s="157"/>
-      <c r="E35" s="158"/>
+      <c r="B35" s="185"/>
+      <c r="C35" s="185"/>
+      <c r="D35" s="202"/>
+      <c r="E35" s="203"/>
       <c r="F35" s="141"/>
       <c r="G35" s="127"/>
       <c r="H35" s="127"/>
       <c r="I35" s="127"/>
       <c r="J35" s="127"/>
       <c r="K35" s="128"/>
-      <c r="L35" s="221"/>
+      <c r="L35" s="193"/>
       <c r="M35" s="148" t="str">
         <f t="shared" ref="M35" si="21">A37</f>
         <v/>
       </c>
-      <c r="N35" s="151" t="str">
+      <c r="N35" s="206" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
-      <c r="O35" s="152"/>
-      <c r="P35" s="219"/>
-      <c r="Q35" s="208"/>
+      <c r="O35" s="207"/>
+      <c r="P35" s="191"/>
+      <c r="Q35" s="212"/>
       <c r="R35" s="150"/>
     </row>
-    <row r="36" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A36" s="134"/>
-      <c r="B36" s="205"/>
-      <c r="C36" s="205"/>
-      <c r="D36" s="155"/>
-      <c r="E36" s="156"/>
+      <c r="B36" s="184"/>
+      <c r="C36" s="184"/>
+      <c r="D36" s="204"/>
+      <c r="E36" s="205"/>
       <c r="F36" s="139"/>
       <c r="G36" s="129"/>
       <c r="H36" s="129"/>
       <c r="I36" s="129"/>
       <c r="J36" s="129"/>
       <c r="K36" s="129"/>
-      <c r="L36" s="221"/>
+      <c r="L36" s="193"/>
       <c r="M36" s="147" t="str">
         <f t="shared" ref="M36" si="22">IF(ISBLANK(A38),"",A38)</f>
         <v/>
       </c>
-      <c r="N36" s="153" t="str">
+      <c r="N36" s="208" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
-      <c r="O36" s="154"/>
-      <c r="P36" s="219"/>
-      <c r="Q36" s="208"/>
+      <c r="O36" s="209"/>
+      <c r="P36" s="191"/>
+      <c r="Q36" s="212"/>
       <c r="R36" s="149"/>
     </row>
-    <row r="37" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A37" s="1" t="str">
         <f t="shared" ref="A37" si="23">IF(A36="","",UPPER(TEXT(A36,"[$-043E]DDDD")))</f>
         <v/>
       </c>
-      <c r="B37" s="206"/>
-      <c r="C37" s="206"/>
-      <c r="D37" s="157"/>
-      <c r="E37" s="158"/>
+      <c r="B37" s="185"/>
+      <c r="C37" s="185"/>
+      <c r="D37" s="202"/>
+      <c r="E37" s="203"/>
       <c r="F37" s="141"/>
       <c r="G37" s="127"/>
       <c r="H37" s="127"/>
       <c r="I37" s="127"/>
       <c r="J37" s="127"/>
       <c r="K37" s="128"/>
-      <c r="L37" s="221"/>
+      <c r="L37" s="193"/>
       <c r="M37" s="148" t="str">
         <f t="shared" ref="M37" si="24">A39</f>
         <v/>
       </c>
-      <c r="N37" s="151" t="str">
+      <c r="N37" s="206" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
-      <c r="O37" s="152"/>
-      <c r="P37" s="219"/>
-      <c r="Q37" s="208"/>
+      <c r="O37" s="207"/>
+      <c r="P37" s="191"/>
+      <c r="Q37" s="212"/>
       <c r="R37" s="150"/>
     </row>
-    <row r="38" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A38" s="134"/>
-      <c r="B38" s="205"/>
-      <c r="C38" s="205"/>
-      <c r="D38" s="155"/>
-      <c r="E38" s="156"/>
+      <c r="B38" s="184"/>
+      <c r="C38" s="184"/>
+      <c r="D38" s="204"/>
+      <c r="E38" s="205"/>
       <c r="F38" s="139"/>
       <c r="G38" s="129"/>
       <c r="H38" s="129"/>
       <c r="I38" s="129"/>
       <c r="J38" s="129"/>
       <c r="K38" s="129"/>
-      <c r="L38" s="221"/>
+      <c r="L38" s="193"/>
       <c r="M38" s="147" t="str">
         <f t="shared" ref="M38" si="25">IF(ISBLANK(A40),"",A40)</f>
         <v/>
       </c>
-      <c r="N38" s="153" t="str">
+      <c r="N38" s="208" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
-      <c r="O38" s="154"/>
-      <c r="P38" s="219"/>
-      <c r="Q38" s="208"/>
+      <c r="O38" s="209"/>
+      <c r="P38" s="191"/>
+      <c r="Q38" s="212"/>
       <c r="R38" s="149"/>
     </row>
-    <row r="39" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A39" s="1" t="str">
         <f t="shared" ref="A39" si="26">IF(A38="","",UPPER(TEXT(A38,"[$-043E]DDDD")))</f>
         <v/>
       </c>
-      <c r="B39" s="206"/>
-      <c r="C39" s="206"/>
-      <c r="D39" s="157"/>
-      <c r="E39" s="158"/>
+      <c r="B39" s="185"/>
+      <c r="C39" s="185"/>
+      <c r="D39" s="202"/>
+      <c r="E39" s="203"/>
       <c r="F39" s="141"/>
       <c r="G39" s="127"/>
       <c r="H39" s="127"/>
       <c r="I39" s="127"/>
       <c r="J39" s="127"/>
       <c r="K39" s="128"/>
-      <c r="L39" s="221"/>
+      <c r="L39" s="193"/>
       <c r="M39" s="148" t="str">
         <f t="shared" ref="M39" si="27">A41</f>
         <v/>
       </c>
-      <c r="N39" s="151" t="str">
+      <c r="N39" s="206" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
-      <c r="O39" s="152"/>
-      <c r="P39" s="219"/>
-      <c r="Q39" s="208"/>
+      <c r="O39" s="207"/>
+      <c r="P39" s="191"/>
+      <c r="Q39" s="212"/>
       <c r="R39" s="150"/>
     </row>
-    <row r="40" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A40" s="134"/>
-      <c r="B40" s="205"/>
-      <c r="C40" s="205"/>
-      <c r="D40" s="155"/>
-      <c r="E40" s="156"/>
+      <c r="B40" s="184"/>
+      <c r="C40" s="184"/>
+      <c r="D40" s="204"/>
+      <c r="E40" s="205"/>
       <c r="F40" s="139"/>
       <c r="G40" s="129"/>
       <c r="H40" s="129"/>
       <c r="I40" s="129"/>
       <c r="J40" s="129"/>
       <c r="K40" s="129"/>
-      <c r="L40" s="221"/>
+      <c r="L40" s="193"/>
       <c r="M40" s="147" t="str">
         <f t="shared" ref="M40" si="28">IF(ISBLANK(A42),"",A42)</f>
         <v/>
       </c>
-      <c r="N40" s="153" t="str">
+      <c r="N40" s="208" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
-      <c r="O40" s="154"/>
-      <c r="P40" s="219"/>
-      <c r="Q40" s="208"/>
+      <c r="O40" s="209"/>
+      <c r="P40" s="191"/>
+      <c r="Q40" s="212"/>
       <c r="R40" s="149"/>
     </row>
-    <row r="41" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A41" s="1" t="str">
         <f t="shared" ref="A41" si="29">IF(A40="","",UPPER(TEXT(A40,"[$-043E]DDDD")))</f>
         <v/>
       </c>
-      <c r="B41" s="206"/>
-      <c r="C41" s="206"/>
-      <c r="D41" s="157"/>
-      <c r="E41" s="158"/>
+      <c r="B41" s="185"/>
+      <c r="C41" s="185"/>
+      <c r="D41" s="202"/>
+      <c r="E41" s="203"/>
       <c r="F41" s="141"/>
       <c r="G41" s="127"/>
       <c r="H41" s="127"/>
       <c r="I41" s="127"/>
       <c r="J41" s="127"/>
       <c r="K41" s="128"/>
-      <c r="L41" s="221"/>
+      <c r="L41" s="193"/>
       <c r="M41" s="148" t="str">
         <f t="shared" ref="M41" si="30">A43</f>
         <v/>
       </c>
-      <c r="N41" s="151" t="str">
+      <c r="N41" s="206" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
-      <c r="O41" s="152"/>
-      <c r="P41" s="219"/>
-      <c r="Q41" s="208"/>
+      <c r="O41" s="207"/>
+      <c r="P41" s="191"/>
+      <c r="Q41" s="212"/>
       <c r="R41" s="150"/>
     </row>
-    <row r="42" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A42" s="134"/>
-      <c r="B42" s="205"/>
-      <c r="C42" s="205"/>
-      <c r="D42" s="155"/>
-      <c r="E42" s="156"/>
+      <c r="B42" s="184"/>
+      <c r="C42" s="184"/>
+      <c r="D42" s="204"/>
+      <c r="E42" s="205"/>
       <c r="F42" s="139"/>
       <c r="G42" s="129"/>
       <c r="H42" s="129"/>
       <c r="I42" s="129"/>
       <c r="J42" s="129"/>
       <c r="K42" s="129"/>
-      <c r="L42" s="221"/>
+      <c r="L42" s="193"/>
       <c r="M42" s="147" t="str">
         <f t="shared" ref="M42" si="31">IF(ISBLANK(A44),"",A44)</f>
         <v/>
       </c>
-      <c r="N42" s="153" t="str">
+      <c r="N42" s="208" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
-      <c r="O42" s="154"/>
-      <c r="P42" s="219"/>
-      <c r="Q42" s="208"/>
+      <c r="O42" s="209"/>
+      <c r="P42" s="191"/>
+      <c r="Q42" s="212"/>
       <c r="R42" s="149"/>
     </row>
-    <row r="43" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A43" s="1" t="str">
         <f t="shared" ref="A43" si="32">IF(A42="","",UPPER(TEXT(A42,"[$-043E]DDDD")))</f>
         <v/>
       </c>
-      <c r="B43" s="206"/>
-      <c r="C43" s="206"/>
-      <c r="D43" s="157"/>
-      <c r="E43" s="158"/>
+      <c r="B43" s="185"/>
+      <c r="C43" s="185"/>
+      <c r="D43" s="202"/>
+      <c r="E43" s="203"/>
       <c r="F43" s="141"/>
       <c r="G43" s="127"/>
       <c r="H43" s="127"/>
       <c r="I43" s="127"/>
       <c r="J43" s="127"/>
       <c r="K43" s="128"/>
-      <c r="L43" s="221"/>
+      <c r="L43" s="193"/>
       <c r="M43" s="148" t="str">
         <f t="shared" ref="M43" si="33">A45</f>
         <v/>
       </c>
-      <c r="N43" s="151" t="str">
+      <c r="N43" s="206" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
-      <c r="O43" s="152"/>
-      <c r="P43" s="219"/>
-      <c r="Q43" s="208"/>
+      <c r="O43" s="207"/>
+      <c r="P43" s="191"/>
+      <c r="Q43" s="212"/>
       <c r="R43" s="150"/>
     </row>
-    <row r="44" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A44" s="134"/>
-      <c r="B44" s="205"/>
-      <c r="C44" s="205"/>
-      <c r="D44" s="155"/>
-      <c r="E44" s="156"/>
+      <c r="B44" s="184"/>
+      <c r="C44" s="184"/>
+      <c r="D44" s="204"/>
+      <c r="E44" s="205"/>
       <c r="F44" s="139"/>
       <c r="G44" s="129"/>
       <c r="H44" s="129"/>
       <c r="I44" s="129"/>
       <c r="J44" s="129"/>
       <c r="K44" s="129"/>
-      <c r="L44" s="221"/>
+      <c r="L44" s="193"/>
       <c r="M44" s="147" t="str">
         <f t="shared" ref="M44" si="34">IF(ISBLANK(A46),"",A46)</f>
         <v/>
       </c>
-      <c r="N44" s="153" t="str">
+      <c r="N44" s="208" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
-      <c r="O44" s="154"/>
-      <c r="P44" s="219"/>
-      <c r="Q44" s="208"/>
+      <c r="O44" s="209"/>
+      <c r="P44" s="191"/>
+      <c r="Q44" s="212"/>
       <c r="R44" s="149"/>
     </row>
-    <row r="45" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A45" s="1" t="str">
         <f t="shared" ref="A45" si="35">IF(A44="","",UPPER(TEXT(A44,"[$-043E]DDDD")))</f>
         <v/>
       </c>
-      <c r="B45" s="206"/>
-      <c r="C45" s="206"/>
-      <c r="D45" s="157"/>
-      <c r="E45" s="158"/>
+      <c r="B45" s="185"/>
+      <c r="C45" s="185"/>
+      <c r="D45" s="202"/>
+      <c r="E45" s="203"/>
       <c r="F45" s="141"/>
       <c r="G45" s="127"/>
       <c r="H45" s="127"/>
       <c r="I45" s="127"/>
       <c r="J45" s="127"/>
       <c r="K45" s="128"/>
-      <c r="L45" s="221"/>
+      <c r="L45" s="193"/>
       <c r="M45" s="148" t="str">
         <f t="shared" ref="M45" si="36">A47</f>
         <v/>
       </c>
-      <c r="N45" s="151" t="str">
+      <c r="N45" s="206" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
-      <c r="O45" s="152"/>
-      <c r="P45" s="219"/>
-      <c r="Q45" s="208"/>
+      <c r="O45" s="207"/>
+      <c r="P45" s="191"/>
+      <c r="Q45" s="212"/>
       <c r="R45" s="150"/>
     </row>
-    <row r="46" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A46" s="134"/>
-      <c r="B46" s="205"/>
-      <c r="C46" s="205"/>
-      <c r="D46" s="155"/>
-      <c r="E46" s="156"/>
+      <c r="B46" s="184"/>
+      <c r="C46" s="184"/>
+      <c r="D46" s="204"/>
+      <c r="E46" s="205"/>
       <c r="F46" s="139"/>
       <c r="G46" s="129"/>
       <c r="H46" s="129"/>
       <c r="I46" s="129"/>
       <c r="J46" s="129"/>
       <c r="K46" s="129"/>
-      <c r="L46" s="221"/>
+      <c r="L46" s="193"/>
       <c r="M46" s="147" t="str">
         <f t="shared" ref="M46" si="37">IF(ISBLANK(A48),"",A48)</f>
         <v/>
       </c>
-      <c r="N46" s="153" t="str">
+      <c r="N46" s="208" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
-      <c r="O46" s="154"/>
-      <c r="P46" s="219"/>
-      <c r="Q46" s="208"/>
+      <c r="O46" s="209"/>
+      <c r="P46" s="191"/>
+      <c r="Q46" s="212"/>
       <c r="R46" s="149"/>
     </row>
-    <row r="47" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A47" s="1" t="str">
         <f t="shared" ref="A47" si="38">IF(A46="","",UPPER(TEXT(A46,"[$-043E]DDDD")))</f>
         <v/>
       </c>
-      <c r="B47" s="206"/>
-      <c r="C47" s="206"/>
-      <c r="D47" s="157"/>
-      <c r="E47" s="158"/>
+      <c r="B47" s="185"/>
+      <c r="C47" s="185"/>
+      <c r="D47" s="202"/>
+      <c r="E47" s="203"/>
       <c r="F47" s="141"/>
       <c r="G47" s="127"/>
       <c r="H47" s="127"/>
       <c r="I47" s="127"/>
       <c r="J47" s="127"/>
       <c r="K47" s="128"/>
-      <c r="L47" s="221"/>
+      <c r="L47" s="193"/>
       <c r="M47" s="148" t="str">
         <f t="shared" ref="M47" si="39">A49</f>
         <v/>
       </c>
-      <c r="N47" s="151" t="str">
+      <c r="N47" s="206" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
-      <c r="O47" s="152"/>
-      <c r="P47" s="219"/>
-      <c r="Q47" s="208"/>
+      <c r="O47" s="207"/>
+      <c r="P47" s="191"/>
+      <c r="Q47" s="212"/>
       <c r="R47" s="150"/>
     </row>
-    <row r="48" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A48" s="134"/>
-      <c r="B48" s="205"/>
-      <c r="C48" s="205"/>
-      <c r="D48" s="155"/>
-      <c r="E48" s="156"/>
+      <c r="B48" s="184"/>
+      <c r="C48" s="184"/>
+      <c r="D48" s="204"/>
+      <c r="E48" s="205"/>
       <c r="F48" s="139"/>
       <c r="G48" s="129"/>
       <c r="H48" s="129"/>
       <c r="I48" s="129"/>
       <c r="J48" s="129"/>
       <c r="K48" s="129"/>
-      <c r="L48" s="221"/>
+      <c r="L48" s="193"/>
       <c r="M48" s="147" t="str">
         <f t="shared" ref="M48" si="40">IF(ISBLANK(A50),"",A50)</f>
         <v/>
       </c>
-      <c r="N48" s="153" t="str">
+      <c r="N48" s="208" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
-      <c r="O48" s="154"/>
-      <c r="P48" s="219"/>
-      <c r="Q48" s="208"/>
+      <c r="O48" s="209"/>
+      <c r="P48" s="191"/>
+      <c r="Q48" s="212"/>
       <c r="R48" s="149"/>
     </row>
-    <row r="49" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A49" s="1" t="str">
         <f t="shared" ref="A49" si="41">IF(A48="","",UPPER(TEXT(A48,"[$-043E]DDDD")))</f>
         <v/>
       </c>
-      <c r="B49" s="206"/>
-      <c r="C49" s="206"/>
-      <c r="D49" s="157"/>
-      <c r="E49" s="158"/>
+      <c r="B49" s="185"/>
+      <c r="C49" s="185"/>
+      <c r="D49" s="202"/>
+      <c r="E49" s="203"/>
       <c r="F49" s="141"/>
       <c r="G49" s="127"/>
       <c r="H49" s="127"/>
       <c r="I49" s="127"/>
       <c r="J49" s="127"/>
       <c r="K49" s="128"/>
-      <c r="L49" s="221"/>
+      <c r="L49" s="193"/>
       <c r="M49" s="148" t="str">
         <f t="shared" ref="M49" si="42">A51</f>
         <v/>
       </c>
-      <c r="N49" s="151" t="str">
+      <c r="N49" s="206" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
-      <c r="O49" s="152"/>
-      <c r="P49" s="219"/>
-      <c r="Q49" s="208"/>
+      <c r="O49" s="207"/>
+      <c r="P49" s="191"/>
+      <c r="Q49" s="212"/>
       <c r="R49" s="150"/>
     </row>
-    <row r="50" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A50" s="134"/>
-      <c r="B50" s="205"/>
-      <c r="C50" s="205"/>
-      <c r="D50" s="155"/>
-      <c r="E50" s="156"/>
+      <c r="B50" s="184"/>
+      <c r="C50" s="184"/>
+      <c r="D50" s="204"/>
+      <c r="E50" s="205"/>
       <c r="F50" s="139"/>
       <c r="G50" s="129"/>
       <c r="H50" s="129"/>
       <c r="I50" s="129"/>
       <c r="J50" s="129"/>
       <c r="K50" s="129"/>
-      <c r="L50" s="221"/>
+      <c r="L50" s="193"/>
       <c r="M50" s="147" t="str">
         <f t="shared" ref="M50" si="43">IF(ISBLANK(A52),"",A52)</f>
         <v/>
       </c>
-      <c r="N50" s="153" t="str">
+      <c r="N50" s="208" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
-      <c r="O50" s="154"/>
-      <c r="P50" s="219"/>
-      <c r="Q50" s="208"/>
+      <c r="O50" s="209"/>
+      <c r="P50" s="191"/>
+      <c r="Q50" s="212"/>
       <c r="R50" s="149"/>
     </row>
-    <row r="51" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A51" s="1" t="str">
         <f t="shared" ref="A51" si="44">IF(A50="","",UPPER(TEXT(A50,"[$-043E]DDDD")))</f>
         <v/>
       </c>
-      <c r="B51" s="206"/>
-      <c r="C51" s="206"/>
-      <c r="D51" s="157"/>
-      <c r="E51" s="158"/>
+      <c r="B51" s="185"/>
+      <c r="C51" s="185"/>
+      <c r="D51" s="202"/>
+      <c r="E51" s="203"/>
       <c r="F51" s="141"/>
       <c r="G51" s="127"/>
       <c r="H51" s="127"/>
       <c r="I51" s="127"/>
       <c r="J51" s="127"/>
       <c r="K51" s="128"/>
-      <c r="L51" s="221"/>
+      <c r="L51" s="193"/>
       <c r="M51" s="148" t="str">
         <f t="shared" ref="M51" si="45">A53</f>
         <v/>
       </c>
-      <c r="N51" s="151" t="str">
+      <c r="N51" s="206" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
-      <c r="O51" s="152"/>
-      <c r="P51" s="219"/>
-      <c r="Q51" s="208"/>
+      <c r="O51" s="207"/>
+      <c r="P51" s="191"/>
+      <c r="Q51" s="212"/>
       <c r="R51" s="150"/>
     </row>
-    <row r="52" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A52" s="134"/>
-      <c r="B52" s="205"/>
-      <c r="C52" s="205"/>
-      <c r="D52" s="155"/>
-      <c r="E52" s="156"/>
+      <c r="B52" s="184"/>
+      <c r="C52" s="184"/>
+      <c r="D52" s="204"/>
+      <c r="E52" s="205"/>
       <c r="F52" s="139"/>
       <c r="G52" s="129"/>
       <c r="H52" s="129"/>
       <c r="I52" s="129"/>
       <c r="J52" s="129"/>
       <c r="K52" s="129"/>
-      <c r="L52" s="221"/>
+      <c r="L52" s="193"/>
       <c r="M52" s="147"/>
-      <c r="N52" s="153" t="str">
+      <c r="N52" s="208" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
-      <c r="O52" s="154"/>
-      <c r="P52" s="219"/>
-      <c r="Q52" s="208"/>
+      <c r="O52" s="209"/>
+      <c r="P52" s="191"/>
+      <c r="Q52" s="212"/>
       <c r="R52" s="149"/>
     </row>
-    <row r="53" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A53" s="1" t="str">
         <f t="shared" ref="A53" si="46">IF(A52="","",UPPER(TEXT(A52,"[$-043E]DDDD")))</f>
         <v/>
       </c>
-      <c r="B53" s="206"/>
-      <c r="C53" s="206"/>
-      <c r="D53" s="157"/>
-      <c r="E53" s="158"/>
+      <c r="B53" s="185"/>
+      <c r="C53" s="185"/>
+      <c r="D53" s="202"/>
+      <c r="E53" s="203"/>
       <c r="F53" s="141"/>
       <c r="G53" s="127"/>
       <c r="H53" s="127"/>
       <c r="I53" s="127"/>
       <c r="J53" s="127"/>
       <c r="K53" s="128"/>
-      <c r="L53" s="222"/>
+      <c r="L53" s="194"/>
       <c r="M53" s="148"/>
-      <c r="N53" s="151" t="str">
+      <c r="N53" s="206" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
-      <c r="O53" s="152"/>
-      <c r="P53" s="220"/>
-      <c r="Q53" s="209"/>
+      <c r="O53" s="207"/>
+      <c r="P53" s="192"/>
+      <c r="Q53" s="213"/>
       <c r="R53" s="150"/>
     </row>
-    <row r="54" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="54" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A54" s="39"/>
       <c r="B54" s="40"/>
       <c r="C54" s="40"/>
@@ -4497,7 +4453,7 @@
       <c r="P54" s="44"/>
       <c r="R54" s="42"/>
     </row>
-    <row r="55" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="55" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A55" s="45"/>
       <c r="B55" s="41"/>
       <c r="C55" s="41"/>
@@ -4528,7 +4484,7 @@
       <c r="O55" s="47"/>
       <c r="P55" s="44"/>
     </row>
-    <row r="56" spans="1:18" ht="15" thickTop="1" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:18" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A56" s="45"/>
       <c r="B56" s="41"/>
       <c r="C56" s="41"/>
@@ -4544,7 +4500,7 @@
       <c r="O56" s="47"/>
       <c r="P56" s="44"/>
     </row>
-    <row r="57" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A57" s="45"/>
       <c r="B57" s="41"/>
       <c r="C57" s="41"/>
@@ -4560,7 +4516,7 @@
       <c r="O57" s="47"/>
       <c r="P57" s="44"/>
     </row>
-    <row r="58" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A58" s="45"/>
       <c r="B58" s="41" t="s">
         <v>28</v>
@@ -4572,8 +4528,8 @@
         <f>SUM(G55:K55)</f>
         <v>0</v>
       </c>
-      <c r="G58" s="210"/>
-      <c r="H58" s="210"/>
+      <c r="G58" s="214"/>
+      <c r="H58" s="214"/>
       <c r="I58" s="49" t="s">
         <v>29</v>
       </c>
@@ -4585,7 +4541,7 @@
       <c r="O58" s="47"/>
       <c r="P58" s="44"/>
     </row>
-    <row r="59" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="59" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A59" s="45"/>
       <c r="B59" s="41" t="s">
         <v>31</v>
@@ -4599,8 +4555,8 @@
         <f>L9</f>
         <v>0</v>
       </c>
-      <c r="G59" s="210"/>
-      <c r="H59" s="210"/>
+      <c r="G59" s="214"/>
+      <c r="H59" s="214"/>
       <c r="I59" s="49"/>
       <c r="J59" s="49"/>
       <c r="K59" s="49"/>
@@ -4608,7 +4564,7 @@
       <c r="O59" s="47"/>
       <c r="P59" s="44"/>
     </row>
-    <row r="60" spans="1:18" ht="15.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="60" spans="1:18" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A60" s="50"/>
       <c r="B60" s="41" t="s">
         <v>33</v>
@@ -4631,7 +4587,7 @@
       <c r="O60" s="47"/>
       <c r="P60" s="44"/>
     </row>
-    <row r="61" spans="1:18" ht="15" thickTop="1" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:18" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A61" s="50"/>
       <c r="B61" s="40"/>
       <c r="C61" s="40"/>
@@ -4647,7 +4603,7 @@
       <c r="O61" s="47"/>
       <c r="P61" s="44"/>
     </row>
-    <row r="62" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A62" s="56"/>
       <c r="B62" s="40" t="s">
         <v>34</v>
@@ -4663,37 +4619,37 @@
       <c r="K62" s="58"/>
       <c r="L62" s="3"/>
     </row>
-    <row r="63" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A63" s="50"/>
       <c r="B63" s="57"/>
-      <c r="C63" s="211" t="s">
+      <c r="C63" s="215" t="s">
         <v>35</v>
       </c>
-      <c r="D63" s="211"/>
-      <c r="E63" s="211"/>
-      <c r="F63" s="211"/>
-      <c r="G63" s="211"/>
-      <c r="H63" s="211"/>
-      <c r="I63" s="211"/>
-      <c r="J63" s="211"/>
-      <c r="K63" s="211"/>
+      <c r="D63" s="215"/>
+      <c r="E63" s="215"/>
+      <c r="F63" s="215"/>
+      <c r="G63" s="215"/>
+      <c r="H63" s="215"/>
+      <c r="I63" s="215"/>
+      <c r="J63" s="215"/>
+      <c r="K63" s="215"/>
       <c r="L63" s="3"/>
     </row>
-    <row r="64" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A64" s="50"/>
       <c r="B64" s="57"/>
-      <c r="C64" s="211"/>
-      <c r="D64" s="211"/>
-      <c r="E64" s="211"/>
-      <c r="F64" s="211"/>
-      <c r="G64" s="211"/>
-      <c r="H64" s="211"/>
-      <c r="I64" s="211"/>
-      <c r="J64" s="211"/>
-      <c r="K64" s="211"/>
+      <c r="C64" s="215"/>
+      <c r="D64" s="215"/>
+      <c r="E64" s="215"/>
+      <c r="F64" s="215"/>
+      <c r="G64" s="215"/>
+      <c r="H64" s="215"/>
+      <c r="I64" s="215"/>
+      <c r="J64" s="215"/>
+      <c r="K64" s="215"/>
       <c r="L64" s="3"/>
     </row>
-    <row r="65" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A65" s="50"/>
       <c r="B65" s="40"/>
       <c r="C65" s="61"/>
@@ -4707,7 +4663,7 @@
       <c r="K65" s="60"/>
       <c r="L65" s="3"/>
     </row>
-    <row r="66" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="66" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A66" s="10"/>
       <c r="B66" s="11"/>
       <c r="C66" s="11"/>
@@ -4724,7 +4680,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="67" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="67" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A67" s="10"/>
       <c r="B67" s="11"/>
       <c r="C67" s="11"/>
@@ -4741,7 +4697,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="68" spans="1:18" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="68" spans="1:18" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A68" s="64" t="s">
         <v>36</v>
       </c>
@@ -4760,7 +4716,7 @@
       <c r="L68" s="3"/>
       <c r="R68" s="65"/>
     </row>
-    <row r="69" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="69" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A69" s="50"/>
       <c r="B69" s="40"/>
       <c r="C69" s="61"/>
@@ -4774,7 +4730,7 @@
       <c r="K69" s="60"/>
       <c r="L69" s="3"/>
     </row>
-    <row r="70" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="70" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A70" s="50"/>
       <c r="B70" s="40"/>
       <c r="C70" s="61"/>
@@ -4788,7 +4744,7 @@
       <c r="K70" s="60"/>
       <c r="L70" s="3"/>
     </row>
-    <row r="71" spans="1:18" ht="20" x14ac:dyDescent="0.35">
+    <row r="71" spans="1:18" ht="20.25" x14ac:dyDescent="0.25">
       <c r="A71" s="50"/>
       <c r="B71" s="40"/>
       <c r="C71" s="61"/>
@@ -4801,16 +4757,16 @@
       <c r="J71" s="60"/>
       <c r="K71" s="60"/>
       <c r="L71" s="3"/>
-      <c r="M71" s="204" t="s">
-        <v>89</v>
-      </c>
-      <c r="N71" s="204"/>
-      <c r="O71" s="204"/>
-      <c r="P71" s="204"/>
-      <c r="Q71" s="204"/>
-      <c r="R71" s="204"/>
-    </row>
-    <row r="72" spans="1:18" ht="20" x14ac:dyDescent="0.35">
+      <c r="M71" s="210" t="s">
+        <v>87</v>
+      </c>
+      <c r="N71" s="210"/>
+      <c r="O71" s="210"/>
+      <c r="P71" s="210"/>
+      <c r="Q71" s="210"/>
+      <c r="R71" s="210"/>
+    </row>
+    <row r="72" spans="1:18" ht="20.25" x14ac:dyDescent="0.25">
       <c r="A72" s="50"/>
       <c r="B72" s="41"/>
       <c r="C72" s="41" t="s">
@@ -4825,20 +4781,20 @@
       <c r="J72" s="60"/>
       <c r="K72" s="60"/>
       <c r="L72" s="3"/>
-      <c r="M72" s="204" t="s">
-        <v>90</v>
-      </c>
-      <c r="N72" s="204"/>
-      <c r="O72" s="204"/>
-      <c r="P72" s="204"/>
-      <c r="Q72" s="204"/>
-      <c r="R72" s="204"/>
-    </row>
-    <row r="73" spans="1:18" ht="16.5" x14ac:dyDescent="0.35">
+      <c r="M72" s="210" t="s">
+        <v>88</v>
+      </c>
+      <c r="N72" s="210"/>
+      <c r="O72" s="210"/>
+      <c r="P72" s="210"/>
+      <c r="Q72" s="210"/>
+      <c r="R72" s="210"/>
+    </row>
+    <row r="73" spans="1:18" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A73" s="50"/>
       <c r="B73" s="66"/>
       <c r="C73" s="66" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="D73" s="67"/>
       <c r="E73" s="68" t="s">
@@ -4851,14 +4807,14 @@
       <c r="J73" s="60"/>
       <c r="K73" s="60"/>
       <c r="L73" s="3"/>
-      <c r="M73" s="196"/>
-      <c r="N73" s="196"/>
-      <c r="O73" s="196"/>
-      <c r="P73" s="196"/>
-      <c r="Q73" s="196"/>
-      <c r="R73" s="196"/>
-    </row>
-    <row r="74" spans="1:18" x14ac:dyDescent="0.35">
+      <c r="M73" s="217"/>
+      <c r="N73" s="217"/>
+      <c r="O73" s="217"/>
+      <c r="P73" s="217"/>
+      <c r="Q73" s="217"/>
+      <c r="R73" s="217"/>
+    </row>
+    <row r="74" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A74" s="50"/>
       <c r="B74" s="40"/>
       <c r="C74" s="40"/>
@@ -4872,7 +4828,7 @@
       <c r="K74" s="60"/>
       <c r="L74" s="3"/>
     </row>
-    <row r="75" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="75" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A75" s="50"/>
       <c r="B75" s="41"/>
       <c r="C75" s="41" t="s">
@@ -4882,26 +4838,26 @@
       <c r="E75" s="68" t="s">
         <v>5</v>
       </c>
-      <c r="F75" s="197">
+      <c r="F75" s="218">
         <f>C8</f>
         <v>0</v>
       </c>
-      <c r="G75" s="197"/>
-      <c r="H75" s="197"/>
-      <c r="I75" s="197"/>
-      <c r="J75" s="197"/>
-      <c r="K75" s="197"/>
+      <c r="G75" s="218"/>
+      <c r="H75" s="218"/>
+      <c r="I75" s="218"/>
+      <c r="J75" s="218"/>
+      <c r="K75" s="218"/>
       <c r="L75" s="3"/>
-      <c r="M75" s="198" t="s">
-        <v>91</v>
-      </c>
-      <c r="N75" s="198"/>
-      <c r="O75" s="198"/>
-      <c r="P75" s="198"/>
-      <c r="Q75" s="198"/>
-      <c r="R75" s="198"/>
-    </row>
-    <row r="76" spans="1:18" ht="18.5" x14ac:dyDescent="0.45">
+      <c r="M75" s="219" t="s">
+        <v>89</v>
+      </c>
+      <c r="N75" s="219"/>
+      <c r="O75" s="219"/>
+      <c r="P75" s="219"/>
+      <c r="Q75" s="219"/>
+      <c r="R75" s="219"/>
+    </row>
+    <row r="76" spans="1:18" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A76" s="50"/>
       <c r="B76" s="40"/>
       <c r="C76" s="40"/>
@@ -4921,7 +4877,7 @@
       <c r="Q76" s="75"/>
       <c r="R76" s="75"/>
     </row>
-    <row r="77" spans="1:18" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="77" spans="1:18" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A77" s="64"/>
       <c r="B77" s="41"/>
       <c r="C77" s="41" t="s">
@@ -4931,14 +4887,14 @@
       <c r="E77" s="68" t="s">
         <v>5</v>
       </c>
-      <c r="F77" s="199">
+      <c r="F77" s="220">
         <f>C10</f>
         <v>0</v>
       </c>
-      <c r="G77" s="199"/>
-      <c r="H77" s="199"/>
-      <c r="I77" s="199"/>
-      <c r="J77" s="199"/>
+      <c r="G77" s="220"/>
+      <c r="H77" s="220"/>
+      <c r="I77" s="220"/>
+      <c r="J77" s="220"/>
       <c r="K77" s="40"/>
       <c r="L77" s="50"/>
       <c r="M77" s="75"/>
@@ -4948,7 +4904,7 @@
       <c r="Q77" s="75"/>
       <c r="R77" s="75"/>
     </row>
-    <row r="78" spans="1:18" ht="18.649999999999999" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="78" spans="1:18" ht="18.600000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A78" s="67"/>
       <c r="B78" s="40"/>
       <c r="C78" s="40"/>
@@ -4963,15 +4919,15 @@
       <c r="L78" s="50"/>
       <c r="M78" s="133"/>
       <c r="N78" s="133"/>
-      <c r="O78" s="201" t="str">
+      <c r="O78" s="222" t="str">
         <f>"NAMA PEGAWAI :    " &amp; C8</f>
         <v xml:space="preserve">NAMA PEGAWAI :    </v>
       </c>
-      <c r="P78" s="201"/>
-      <c r="Q78" s="201"/>
-      <c r="R78" s="201"/>
-    </row>
-    <row r="79" spans="1:18" ht="18.5" x14ac:dyDescent="0.35">
+      <c r="P78" s="222"/>
+      <c r="Q78" s="222"/>
+      <c r="R78" s="222"/>
+    </row>
+    <row r="79" spans="1:18" ht="18.75" x14ac:dyDescent="0.25">
       <c r="A79" s="67"/>
       <c r="B79" s="40"/>
       <c r="C79" s="40" t="s">
@@ -4991,14 +4947,14 @@
       <c r="M79" s="77"/>
       <c r="N79" s="77"/>
       <c r="O79" s="78"/>
-      <c r="P79" s="200" t="str">
+      <c r="P79" s="221" t="str">
         <f>"                      "&amp;C11</f>
         <v xml:space="preserve">                      </v>
       </c>
-      <c r="Q79" s="200"/>
+      <c r="Q79" s="221"/>
       <c r="R79" s="79"/>
     </row>
-    <row r="80" spans="1:18" ht="18.5" x14ac:dyDescent="0.35">
+    <row r="80" spans="1:18" ht="18.75" x14ac:dyDescent="0.25">
       <c r="A80" s="50"/>
       <c r="B80" s="67"/>
       <c r="C80" s="40"/>
@@ -5018,7 +4974,7 @@
       <c r="Q80" s="78"/>
       <c r="R80" s="80"/>
     </row>
-    <row r="81" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="81" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A81" s="50"/>
       <c r="B81" s="67"/>
       <c r="C81" s="41"/>
@@ -5033,15 +4989,15 @@
       <c r="L81" s="50"/>
       <c r="M81" s="78"/>
       <c r="N81" s="78"/>
-      <c r="O81" s="202" t="str">
+      <c r="O81" s="223" t="str">
         <f>"NO. PEGAWAI :        " &amp; C10</f>
         <v xml:space="preserve">NO. PEGAWAI :        </v>
       </c>
-      <c r="P81" s="202"/>
-      <c r="Q81" s="202"/>
-      <c r="R81" s="202"/>
-    </row>
-    <row r="82" spans="1:18" ht="18.5" x14ac:dyDescent="0.45">
+      <c r="P81" s="223"/>
+      <c r="Q81" s="223"/>
+      <c r="R81" s="223"/>
+    </row>
+    <row r="82" spans="1:18" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A82" s="50"/>
       <c r="B82" s="67"/>
       <c r="C82" s="66"/>
@@ -5061,7 +5017,7 @@
       <c r="Q82" s="75"/>
       <c r="R82" s="75"/>
     </row>
-    <row r="83" spans="1:18" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="83" spans="1:18" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A83" s="50"/>
       <c r="B83" s="67"/>
       <c r="C83" s="41" t="s">
@@ -5076,18 +5032,18 @@
       <c r="J83" s="50"/>
       <c r="K83" s="50"/>
       <c r="L83" s="50"/>
-      <c r="M83" s="203"/>
-      <c r="N83" s="203"/>
-      <c r="O83" s="203"/>
-      <c r="P83" s="203"/>
-      <c r="Q83" s="203"/>
-      <c r="R83" s="203"/>
-    </row>
-    <row r="84" spans="1:18" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="M83" s="224"/>
+      <c r="N83" s="224"/>
+      <c r="O83" s="224"/>
+      <c r="P83" s="224"/>
+      <c r="Q83" s="224"/>
+      <c r="R83" s="224"/>
+    </row>
+    <row r="84" spans="1:18" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A84" s="50"/>
       <c r="B84" s="67"/>
       <c r="C84" s="66" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="D84" s="50"/>
       <c r="E84" s="68" t="s">
@@ -5100,16 +5056,16 @@
       <c r="J84" s="74"/>
       <c r="K84" s="50"/>
       <c r="L84" s="50"/>
-      <c r="M84" s="182" t="s">
-        <v>92</v>
-      </c>
-      <c r="N84" s="182"/>
-      <c r="O84" s="182"/>
-      <c r="P84" s="182"/>
-      <c r="Q84" s="182"/>
-      <c r="R84" s="182"/>
-    </row>
-    <row r="85" spans="1:18" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="M84" s="216" t="s">
+        <v>90</v>
+      </c>
+      <c r="N84" s="216"/>
+      <c r="O84" s="216"/>
+      <c r="P84" s="216"/>
+      <c r="Q84" s="216"/>
+      <c r="R84" s="216"/>
+    </row>
+    <row r="85" spans="1:18" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A85" s="50"/>
       <c r="B85" s="67"/>
       <c r="C85" s="40"/>
@@ -5122,16 +5078,16 @@
       <c r="J85" s="50"/>
       <c r="K85" s="50"/>
       <c r="L85" s="50"/>
-      <c r="M85" s="182" t="s">
-        <v>93</v>
-      </c>
-      <c r="N85" s="182"/>
-      <c r="O85" s="182"/>
-      <c r="P85" s="182"/>
-      <c r="Q85" s="182"/>
-      <c r="R85" s="182"/>
-    </row>
-    <row r="86" spans="1:18" ht="18" x14ac:dyDescent="0.4">
+      <c r="M85" s="216" t="s">
+        <v>91</v>
+      </c>
+      <c r="N85" s="216"/>
+      <c r="O85" s="216"/>
+      <c r="P85" s="216"/>
+      <c r="Q85" s="216"/>
+      <c r="R85" s="216"/>
+    </row>
+    <row r="86" spans="1:18" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A86" s="50"/>
       <c r="B86" s="67"/>
       <c r="C86" s="41" t="s">
@@ -5148,14 +5104,14 @@
       <c r="J86" s="50"/>
       <c r="K86" s="50"/>
       <c r="L86" s="50"/>
-      <c r="M86" s="183"/>
-      <c r="N86" s="183"/>
-      <c r="O86" s="183"/>
-      <c r="P86" s="183"/>
-      <c r="Q86" s="183"/>
-      <c r="R86" s="183"/>
-    </row>
-    <row r="87" spans="1:18" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="M86" s="225"/>
+      <c r="N86" s="225"/>
+      <c r="O86" s="225"/>
+      <c r="P86" s="225"/>
+      <c r="Q86" s="225"/>
+      <c r="R86" s="225"/>
+    </row>
+    <row r="87" spans="1:18" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A87" s="50"/>
       <c r="B87" s="67"/>
       <c r="C87" s="40"/>
@@ -5168,14 +5124,14 @@
       <c r="J87" s="50"/>
       <c r="K87" s="50"/>
       <c r="L87" s="50"/>
-      <c r="M87" s="182"/>
-      <c r="N87" s="182"/>
-      <c r="O87" s="182"/>
-      <c r="P87" s="182"/>
-      <c r="Q87" s="182"/>
-      <c r="R87" s="182"/>
-    </row>
-    <row r="88" spans="1:18" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="M87" s="216"/>
+      <c r="N87" s="216"/>
+      <c r="O87" s="216"/>
+      <c r="P87" s="216"/>
+      <c r="Q87" s="216"/>
+      <c r="R87" s="216"/>
+    </row>
+    <row r="88" spans="1:18" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A88" s="50"/>
       <c r="B88" s="67"/>
       <c r="C88" s="41" t="s">
@@ -5185,23 +5141,23 @@
       <c r="E88" s="68" t="s">
         <v>5</v>
       </c>
-      <c r="F88" s="181"/>
-      <c r="G88" s="181"/>
-      <c r="H88" s="181"/>
-      <c r="I88" s="181"/>
-      <c r="J88" s="181"/>
+      <c r="F88" s="240"/>
+      <c r="G88" s="240"/>
+      <c r="H88" s="240"/>
+      <c r="I88" s="240"/>
+      <c r="J88" s="240"/>
       <c r="K88" s="50"/>
       <c r="L88" s="50"/>
-      <c r="M88" s="182" t="s">
-        <v>94</v>
-      </c>
-      <c r="N88" s="182"/>
-      <c r="O88" s="182"/>
-      <c r="P88" s="182"/>
-      <c r="Q88" s="182"/>
-      <c r="R88" s="182"/>
-    </row>
-    <row r="89" spans="1:18" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="M88" s="216" t="s">
+        <v>92</v>
+      </c>
+      <c r="N88" s="216"/>
+      <c r="O88" s="216"/>
+      <c r="P88" s="216"/>
+      <c r="Q88" s="216"/>
+      <c r="R88" s="216"/>
+    </row>
+    <row r="89" spans="1:18" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A89" s="50"/>
       <c r="B89" s="67"/>
       <c r="C89" s="40"/>
@@ -5215,7 +5171,7 @@
       <c r="K89" s="50"/>
       <c r="L89" s="50"/>
       <c r="M89" s="83" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="N89" s="83"/>
       <c r="O89" s="83"/>
@@ -5223,7 +5179,7 @@
       <c r="Q89" s="83"/>
       <c r="R89" s="83"/>
     </row>
-    <row r="90" spans="1:18" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="90" spans="1:18" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A90" s="50"/>
       <c r="B90" s="67"/>
       <c r="C90" s="40" t="s">
@@ -5247,7 +5203,7 @@
       <c r="Q90" s="83"/>
       <c r="R90" s="83"/>
     </row>
-    <row r="91" spans="1:18" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="91" spans="1:18" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A91" s="50"/>
       <c r="B91" s="67"/>
       <c r="C91" s="41"/>
@@ -5261,7 +5217,7 @@
       <c r="K91" s="50"/>
       <c r="L91" s="50"/>
       <c r="M91" s="83" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="N91" s="83"/>
       <c r="O91" s="83"/>
@@ -5269,7 +5225,7 @@
       <c r="Q91" s="83"/>
       <c r="R91" s="83"/>
     </row>
-    <row r="92" spans="1:18" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="92" spans="1:18" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A92" s="50"/>
       <c r="B92" s="67"/>
       <c r="C92" s="40"/>
@@ -5289,7 +5245,7 @@
       <c r="Q92" s="83"/>
       <c r="R92" s="83"/>
     </row>
-    <row r="93" spans="1:18" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="93" spans="1:18" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A93" s="50"/>
       <c r="B93" s="67"/>
       <c r="C93" s="40"/>
@@ -5303,7 +5259,7 @@
       <c r="K93" s="50"/>
       <c r="L93" s="50"/>
       <c r="M93" s="83" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="N93" s="83"/>
       <c r="O93" s="83"/>
@@ -5311,7 +5267,7 @@
       <c r="Q93" s="83"/>
       <c r="R93" s="83"/>
     </row>
-    <row r="94" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="94" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A94" s="64" t="s">
         <v>44</v>
       </c>
@@ -5329,7 +5285,7 @@
       <c r="K94" s="27"/>
       <c r="L94" s="17"/>
       <c r="M94" s="83" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="N94" s="83"/>
       <c r="O94" s="83"/>
@@ -5337,7 +5293,7 @@
       <c r="Q94" s="83"/>
       <c r="R94" s="83"/>
     </row>
-    <row r="95" spans="1:18" ht="18" x14ac:dyDescent="0.4">
+    <row r="95" spans="1:18" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A95" s="64"/>
       <c r="B95" s="86" t="s">
         <v>46</v>
@@ -5352,14 +5308,14 @@
       <c r="J95" s="86"/>
       <c r="K95" s="27"/>
       <c r="L95" s="17"/>
-      <c r="M95" s="183"/>
-      <c r="N95" s="183"/>
-      <c r="O95" s="183"/>
-      <c r="P95" s="183"/>
-      <c r="Q95" s="183"/>
-      <c r="R95" s="183"/>
-    </row>
-    <row r="96" spans="1:18" ht="18" x14ac:dyDescent="0.4">
+      <c r="M95" s="225"/>
+      <c r="N95" s="225"/>
+      <c r="O95" s="225"/>
+      <c r="P95" s="225"/>
+      <c r="Q95" s="225"/>
+      <c r="R95" s="225"/>
+    </row>
+    <row r="96" spans="1:18" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A96" s="64"/>
       <c r="B96" s="86" t="s">
         <v>47</v>
@@ -5374,14 +5330,14 @@
       <c r="J96" s="86"/>
       <c r="K96" s="27"/>
       <c r="L96" s="17"/>
-      <c r="M96" s="183"/>
-      <c r="N96" s="183"/>
-      <c r="O96" s="183"/>
-      <c r="P96" s="183"/>
-      <c r="Q96" s="183"/>
-      <c r="R96" s="183"/>
-    </row>
-    <row r="97" spans="1:18" ht="18" x14ac:dyDescent="0.4">
+      <c r="M96" s="225"/>
+      <c r="N96" s="225"/>
+      <c r="O96" s="225"/>
+      <c r="P96" s="225"/>
+      <c r="Q96" s="225"/>
+      <c r="R96" s="225"/>
+    </row>
+    <row r="97" spans="1:18" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A97" s="64"/>
       <c r="B97" s="86" t="s">
         <v>48</v>
@@ -5396,14 +5352,14 @@
       <c r="J97" s="86"/>
       <c r="K97" s="27"/>
       <c r="L97" s="17"/>
-      <c r="M97" s="183"/>
-      <c r="N97" s="183"/>
-      <c r="O97" s="183"/>
-      <c r="P97" s="183"/>
-      <c r="Q97" s="183"/>
-      <c r="R97" s="183"/>
-    </row>
-    <row r="98" spans="1:18" ht="18" x14ac:dyDescent="0.4">
+      <c r="M97" s="225"/>
+      <c r="N97" s="225"/>
+      <c r="O97" s="225"/>
+      <c r="P97" s="225"/>
+      <c r="Q97" s="225"/>
+      <c r="R97" s="225"/>
+    </row>
+    <row r="98" spans="1:18" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A98" s="64"/>
       <c r="B98" s="86" t="s">
         <v>49</v>
@@ -5418,14 +5374,14 @@
       <c r="J98" s="86"/>
       <c r="K98" s="27"/>
       <c r="L98" s="17"/>
-      <c r="M98" s="183"/>
-      <c r="N98" s="183"/>
-      <c r="O98" s="183"/>
-      <c r="P98" s="183"/>
-      <c r="Q98" s="183"/>
-      <c r="R98" s="183"/>
-    </row>
-    <row r="99" spans="1:18" x14ac:dyDescent="0.35">
+      <c r="M98" s="225"/>
+      <c r="N98" s="225"/>
+      <c r="O98" s="225"/>
+      <c r="P98" s="225"/>
+      <c r="Q98" s="225"/>
+      <c r="R98" s="225"/>
+    </row>
+    <row r="99" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A99" s="64"/>
       <c r="B99" s="86" t="s">
         <v>50</v>
@@ -5440,14 +5396,14 @@
       <c r="J99" s="27"/>
       <c r="K99" s="27"/>
       <c r="L99" s="17"/>
-      <c r="M99" s="182"/>
-      <c r="N99" s="182"/>
-      <c r="O99" s="182"/>
-      <c r="P99" s="182"/>
-      <c r="Q99" s="182"/>
-      <c r="R99" s="182"/>
-    </row>
-    <row r="100" spans="1:18" x14ac:dyDescent="0.35">
+      <c r="M99" s="216"/>
+      <c r="N99" s="216"/>
+      <c r="O99" s="216"/>
+      <c r="P99" s="216"/>
+      <c r="Q99" s="216"/>
+      <c r="R99" s="216"/>
+    </row>
+    <row r="100" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A100" s="50"/>
       <c r="B100" s="86"/>
       <c r="C100" s="18"/>
@@ -5467,7 +5423,7 @@
       <c r="Q100" s="83"/>
       <c r="R100" s="83"/>
     </row>
-    <row r="101" spans="1:18" ht="18.5" x14ac:dyDescent="0.35">
+    <row r="101" spans="1:18" ht="18.75" x14ac:dyDescent="0.25">
       <c r="A101" s="64" t="s">
         <v>51</v>
       </c>
@@ -5486,7 +5442,7 @@
       <c r="L101" s="17"/>
       <c r="O101" s="79"/>
     </row>
-    <row r="102" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="102" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A102" s="64"/>
       <c r="B102" s="18" t="s">
         <v>53</v>
@@ -5502,7 +5458,7 @@
       <c r="K102" s="17"/>
       <c r="L102" s="17"/>
     </row>
-    <row r="103" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="103" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A103" s="64"/>
       <c r="B103" s="18" t="s">
         <v>54</v>
@@ -5518,10 +5474,10 @@
       <c r="K103" s="17"/>
       <c r="L103" s="17"/>
       <c r="O103" s="77" t="s">
-        <v>105</v>
-      </c>
-    </row>
-    <row r="104" spans="1:18" x14ac:dyDescent="0.35">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="104" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A104" s="64"/>
       <c r="B104" s="41"/>
       <c r="C104" s="92"/>
@@ -5538,7 +5494,7 @@
       <c r="Q104" s="94"/>
       <c r="R104" s="94"/>
     </row>
-    <row r="105" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="105" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A105" s="64"/>
       <c r="B105" s="40" t="s">
         <v>55</v>
@@ -5554,7 +5510,7 @@
       <c r="K105" s="50"/>
       <c r="L105" s="50"/>
     </row>
-    <row r="106" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="106" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A106" s="64"/>
       <c r="B106" s="40"/>
       <c r="C106" s="95"/>
@@ -5568,7 +5524,7 @@
       <c r="K106" s="50"/>
       <c r="L106" s="50"/>
     </row>
-    <row r="107" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="107" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A107" s="64"/>
       <c r="B107" s="40"/>
       <c r="C107" s="95"/>
@@ -5582,19 +5538,19 @@
       <c r="K107" s="50"/>
       <c r="L107" s="50"/>
       <c r="O107" s="94" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="P107" s="94"/>
       <c r="Q107" s="94"/>
       <c r="R107" s="94"/>
     </row>
-    <row r="108" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="108" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A108" s="64" t="s">
         <v>56</v>
       </c>
       <c r="B108" s="95"/>
       <c r="C108" s="40" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="D108" s="40"/>
       <c r="E108" s="68" t="s">
@@ -5611,7 +5567,7 @@
       <c r="Q108" s="94"/>
       <c r="R108" s="94"/>
     </row>
-    <row r="109" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="109" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A109" s="55"/>
       <c r="B109" s="95"/>
       <c r="C109" s="40"/>
@@ -5625,13 +5581,13 @@
       <c r="K109" s="50"/>
       <c r="L109" s="50"/>
       <c r="O109" s="83" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="P109" s="94"/>
       <c r="Q109" s="94"/>
       <c r="R109" s="94"/>
     </row>
-    <row r="110" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="110" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A110" s="50"/>
       <c r="B110" s="95"/>
       <c r="C110" s="41" t="s">
@@ -5649,10 +5605,10 @@
       <c r="K110" s="50"/>
       <c r="L110" s="50"/>
       <c r="O110" s="99" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="111" spans="1:18" x14ac:dyDescent="0.35">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="111" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A111" s="50"/>
       <c r="B111" s="95"/>
       <c r="C111" s="66"/>
@@ -5666,13 +5622,13 @@
       <c r="K111" s="50"/>
       <c r="L111" s="50"/>
       <c r="O111" s="99" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="P111" s="94"/>
       <c r="Q111" s="94"/>
       <c r="R111" s="94"/>
     </row>
-    <row r="112" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="112" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A112" s="50"/>
       <c r="B112" s="95"/>
       <c r="C112" s="41" t="s">
@@ -5690,12 +5646,12 @@
       <c r="K112" s="50"/>
       <c r="L112" s="50"/>
       <c r="O112" s="99" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="Q112" s="100"/>
       <c r="R112" s="100"/>
     </row>
-    <row r="113" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="113" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A113" s="50"/>
       <c r="B113" s="95"/>
       <c r="C113" s="40"/>
@@ -5713,7 +5669,7 @@
       <c r="Q113" s="94"/>
       <c r="R113" s="94"/>
     </row>
-    <row r="114" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="114" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A114" s="17"/>
       <c r="B114" s="91"/>
       <c r="C114" s="86" t="s">
@@ -5731,78 +5687,78 @@
       <c r="K114" s="17"/>
       <c r="L114" s="50"/>
       <c r="O114" s="99" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="P114" s="8" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="115" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="115" spans="1:18" x14ac:dyDescent="0.25">
       <c r="O115" s="83"/>
     </row>
-    <row r="116" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="116" spans="1:18" x14ac:dyDescent="0.25">
       <c r="O116" s="99" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="P116" s="8" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="119" spans="1:18" ht="60" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="124" spans="1:18" ht="18.5" x14ac:dyDescent="0.35">
-      <c r="A124" s="184" t="s">
+    <row r="119" spans="1:18" ht="60" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="124" spans="1:18" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="A124" s="241" t="s">
         <v>65</v>
       </c>
-      <c r="B124" s="185"/>
-      <c r="C124" s="185"/>
-      <c r="D124" s="185"/>
-      <c r="E124" s="185"/>
-      <c r="F124" s="185"/>
-      <c r="G124" s="185"/>
-      <c r="H124" s="185"/>
-      <c r="I124" s="185"/>
-      <c r="J124" s="185"/>
-      <c r="K124" s="185"/>
-      <c r="L124" s="186"/>
-    </row>
-    <row r="125" spans="1:18" ht="27" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A125" s="187" t="s">
+      <c r="B124" s="242"/>
+      <c r="C124" s="242"/>
+      <c r="D124" s="242"/>
+      <c r="E124" s="242"/>
+      <c r="F124" s="242"/>
+      <c r="G124" s="242"/>
+      <c r="H124" s="242"/>
+      <c r="I124" s="242"/>
+      <c r="J124" s="242"/>
+      <c r="K124" s="242"/>
+      <c r="L124" s="243"/>
+    </row>
+    <row r="125" spans="1:18" ht="27" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A125" s="244" t="s">
         <v>66</v>
       </c>
-      <c r="B125" s="188"/>
-      <c r="C125" s="188"/>
-      <c r="D125" s="188"/>
-      <c r="E125" s="188"/>
-      <c r="F125" s="188"/>
-      <c r="G125" s="188"/>
-      <c r="H125" s="188"/>
-      <c r="I125" s="188"/>
-      <c r="J125" s="188"/>
-      <c r="K125" s="188"/>
-      <c r="L125" s="189"/>
-    </row>
-    <row r="126" spans="1:18" ht="27" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B125" s="245"/>
+      <c r="C125" s="245"/>
+      <c r="D125" s="245"/>
+      <c r="E125" s="245"/>
+      <c r="F125" s="245"/>
+      <c r="G125" s="245"/>
+      <c r="H125" s="245"/>
+      <c r="I125" s="245"/>
+      <c r="J125" s="245"/>
+      <c r="K125" s="245"/>
+      <c r="L125" s="246"/>
+    </row>
+    <row r="126" spans="1:18" ht="27" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A126" s="105" t="s">
         <v>67</v>
       </c>
       <c r="B126" s="106"/>
       <c r="C126" s="106"/>
-      <c r="D126" s="190">
+      <c r="D126" s="247">
         <f>C8</f>
         <v>0</v>
       </c>
-      <c r="E126" s="191"/>
-      <c r="F126" s="191"/>
-      <c r="G126" s="191"/>
-      <c r="H126" s="191"/>
-      <c r="I126" s="192"/>
-      <c r="J126" s="193" t="s">
+      <c r="E126" s="248"/>
+      <c r="F126" s="248"/>
+      <c r="G126" s="248"/>
+      <c r="H126" s="248"/>
+      <c r="I126" s="249"/>
+      <c r="J126" s="250" t="s">
         <v>68</v>
       </c>
-      <c r="K126" s="194"/>
-      <c r="L126" s="195"/>
-    </row>
-    <row r="127" spans="1:18" ht="27" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="K126" s="251"/>
+      <c r="L126" s="252"/>
+    </row>
+    <row r="127" spans="1:18" ht="27" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A127" s="107" t="s">
         <v>69</v>
       </c>
@@ -5818,7 +5774,7 @@
       <c r="K127" s="112"/>
       <c r="L127" s="113"/>
     </row>
-    <row r="128" spans="1:18" ht="38.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="128" spans="1:18" ht="38.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A128" s="114"/>
       <c r="B128" s="115"/>
       <c r="C128" s="115"/>
@@ -5832,29 +5788,29 @@
       <c r="K128" s="118"/>
       <c r="L128" s="119"/>
     </row>
-    <row r="129" spans="1:12" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="129" spans="1:12" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A129" s="120" t="s">
         <v>70</v>
       </c>
-      <c r="B129" s="171" t="s">
+      <c r="B129" s="230" t="s">
         <v>71</v>
       </c>
-      <c r="C129" s="172"/>
-      <c r="D129" s="173" t="s">
+      <c r="C129" s="231"/>
+      <c r="D129" s="232" t="s">
         <v>72</v>
       </c>
-      <c r="E129" s="174"/>
-      <c r="F129" s="174"/>
-      <c r="G129" s="174"/>
-      <c r="H129" s="174"/>
-      <c r="I129" s="174"/>
-      <c r="J129" s="175"/>
-      <c r="K129" s="173" t="s">
+      <c r="E129" s="233"/>
+      <c r="F129" s="233"/>
+      <c r="G129" s="233"/>
+      <c r="H129" s="233"/>
+      <c r="I129" s="233"/>
+      <c r="J129" s="234"/>
+      <c r="K129" s="232" t="s">
         <v>73</v>
       </c>
-      <c r="L129" s="174"/>
-    </row>
-    <row r="130" spans="1:12" ht="42" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="L129" s="233"/>
+    </row>
+    <row r="130" spans="1:12" ht="42" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A130" s="121"/>
       <c r="B130" s="122" t="s">
         <v>74</v>
@@ -5862,243 +5818,349 @@
       <c r="C130" s="123" t="s">
         <v>75</v>
       </c>
-      <c r="D130" s="176"/>
-      <c r="E130" s="177"/>
-      <c r="F130" s="177"/>
-      <c r="G130" s="177"/>
-      <c r="H130" s="177"/>
-      <c r="I130" s="177"/>
-      <c r="J130" s="178"/>
-      <c r="K130" s="179"/>
-      <c r="L130" s="180"/>
-    </row>
-    <row r="131" spans="1:12" ht="42" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="D130" s="235"/>
+      <c r="E130" s="236"/>
+      <c r="F130" s="236"/>
+      <c r="G130" s="236"/>
+      <c r="H130" s="236"/>
+      <c r="I130" s="236"/>
+      <c r="J130" s="237"/>
+      <c r="K130" s="238"/>
+      <c r="L130" s="239"/>
+    </row>
+    <row r="131" spans="1:12" ht="42" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A131" s="124">
         <v>1</v>
       </c>
       <c r="B131" s="124"/>
       <c r="C131" s="125"/>
-      <c r="D131" s="166" t="s">
+      <c r="D131" s="227" t="s">
         <v>76</v>
       </c>
-      <c r="E131" s="167"/>
-      <c r="F131" s="167"/>
-      <c r="G131" s="167"/>
-      <c r="H131" s="167"/>
-      <c r="I131" s="167"/>
-      <c r="J131" s="168"/>
-      <c r="K131" s="162"/>
-      <c r="L131" s="162"/>
-    </row>
-    <row r="132" spans="1:12" ht="42" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="E131" s="228"/>
+      <c r="F131" s="228"/>
+      <c r="G131" s="228"/>
+      <c r="H131" s="228"/>
+      <c r="I131" s="228"/>
+      <c r="J131" s="229"/>
+      <c r="K131" s="226"/>
+      <c r="L131" s="226"/>
+    </row>
+    <row r="132" spans="1:12" ht="42" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A132" s="124">
         <v>2</v>
       </c>
       <c r="B132" s="124"/>
       <c r="C132" s="126"/>
-      <c r="D132" s="166" t="s">
+      <c r="D132" s="227" t="s">
         <v>77</v>
       </c>
-      <c r="E132" s="167"/>
-      <c r="F132" s="167"/>
-      <c r="G132" s="167"/>
-      <c r="H132" s="167"/>
-      <c r="I132" s="167"/>
-      <c r="J132" s="168"/>
-      <c r="K132" s="162"/>
-      <c r="L132" s="162"/>
-    </row>
-    <row r="133" spans="1:12" ht="42" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="E132" s="228"/>
+      <c r="F132" s="228"/>
+      <c r="G132" s="228"/>
+      <c r="H132" s="228"/>
+      <c r="I132" s="228"/>
+      <c r="J132" s="229"/>
+      <c r="K132" s="226"/>
+      <c r="L132" s="226"/>
+    </row>
+    <row r="133" spans="1:12" ht="42" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A133" s="124">
         <v>3</v>
       </c>
       <c r="B133" s="124"/>
       <c r="C133" s="126"/>
-      <c r="D133" s="166" t="s">
+      <c r="D133" s="227" t="s">
         <v>78</v>
       </c>
-      <c r="E133" s="167"/>
-      <c r="F133" s="167"/>
-      <c r="G133" s="167"/>
-      <c r="H133" s="167"/>
-      <c r="I133" s="167"/>
-      <c r="J133" s="168"/>
-      <c r="K133" s="162"/>
-      <c r="L133" s="162"/>
-    </row>
-    <row r="134" spans="1:12" ht="42" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="E133" s="228"/>
+      <c r="F133" s="228"/>
+      <c r="G133" s="228"/>
+      <c r="H133" s="228"/>
+      <c r="I133" s="228"/>
+      <c r="J133" s="229"/>
+      <c r="K133" s="226"/>
+      <c r="L133" s="226"/>
+    </row>
+    <row r="134" spans="1:12" ht="42" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A134" s="124">
         <v>4</v>
       </c>
       <c r="B134" s="124"/>
       <c r="C134" s="126"/>
-      <c r="D134" s="166" t="s">
+      <c r="D134" s="227" t="s">
         <v>79</v>
       </c>
-      <c r="E134" s="167"/>
-      <c r="F134" s="167"/>
-      <c r="G134" s="167"/>
-      <c r="H134" s="167"/>
-      <c r="I134" s="167"/>
-      <c r="J134" s="168"/>
-      <c r="K134" s="162"/>
-      <c r="L134" s="162"/>
-    </row>
-    <row r="135" spans="1:12" ht="42" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="E134" s="228"/>
+      <c r="F134" s="228"/>
+      <c r="G134" s="228"/>
+      <c r="H134" s="228"/>
+      <c r="I134" s="228"/>
+      <c r="J134" s="229"/>
+      <c r="K134" s="226"/>
+      <c r="L134" s="226"/>
+    </row>
+    <row r="135" spans="1:12" ht="42" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A135" s="124">
         <v>5</v>
       </c>
       <c r="B135" s="124"/>
       <c r="C135" s="126"/>
-      <c r="D135" s="166" t="s">
+      <c r="D135" s="227" t="s">
         <v>80</v>
       </c>
-      <c r="E135" s="167"/>
-      <c r="F135" s="167"/>
-      <c r="G135" s="167"/>
-      <c r="H135" s="167"/>
-      <c r="I135" s="167"/>
-      <c r="J135" s="168"/>
-      <c r="K135" s="162"/>
-      <c r="L135" s="162"/>
-    </row>
-    <row r="136" spans="1:12" ht="42" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="E135" s="228"/>
+      <c r="F135" s="228"/>
+      <c r="G135" s="228"/>
+      <c r="H135" s="228"/>
+      <c r="I135" s="228"/>
+      <c r="J135" s="229"/>
+      <c r="K135" s="226"/>
+      <c r="L135" s="226"/>
+    </row>
+    <row r="136" spans="1:12" ht="42" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A136" s="124">
         <v>6</v>
       </c>
       <c r="B136" s="124"/>
       <c r="C136" s="126"/>
-      <c r="D136" s="166" t="s">
+      <c r="D136" s="227" t="s">
         <v>81</v>
       </c>
-      <c r="E136" s="167"/>
-      <c r="F136" s="167"/>
-      <c r="G136" s="167"/>
-      <c r="H136" s="167"/>
-      <c r="I136" s="167"/>
-      <c r="J136" s="168"/>
-      <c r="K136" s="162"/>
-      <c r="L136" s="162"/>
-    </row>
-    <row r="137" spans="1:12" ht="42" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="E136" s="228"/>
+      <c r="F136" s="228"/>
+      <c r="G136" s="228"/>
+      <c r="H136" s="228"/>
+      <c r="I136" s="228"/>
+      <c r="J136" s="229"/>
+      <c r="K136" s="226"/>
+      <c r="L136" s="226"/>
+    </row>
+    <row r="137" spans="1:12" ht="42" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A137" s="124">
         <v>7</v>
       </c>
       <c r="B137" s="124"/>
       <c r="C137" s="126"/>
-      <c r="D137" s="166" t="s">
+      <c r="D137" s="227" t="s">
         <v>82</v>
       </c>
-      <c r="E137" s="167"/>
-      <c r="F137" s="167"/>
-      <c r="G137" s="167"/>
-      <c r="H137" s="167"/>
-      <c r="I137" s="167"/>
-      <c r="J137" s="168"/>
-      <c r="K137" s="162"/>
-      <c r="L137" s="162"/>
-    </row>
-    <row r="138" spans="1:12" ht="42" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="E137" s="228"/>
+      <c r="F137" s="228"/>
+      <c r="G137" s="228"/>
+      <c r="H137" s="228"/>
+      <c r="I137" s="228"/>
+      <c r="J137" s="229"/>
+      <c r="K137" s="226"/>
+      <c r="L137" s="226"/>
+    </row>
+    <row r="138" spans="1:12" ht="42" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A138" s="124">
         <v>8</v>
       </c>
       <c r="B138" s="124"/>
       <c r="C138" s="126"/>
-      <c r="D138" s="159" t="s">
-        <v>111</v>
-      </c>
-      <c r="E138" s="160"/>
-      <c r="F138" s="160"/>
-      <c r="G138" s="160"/>
-      <c r="H138" s="160"/>
-      <c r="I138" s="160"/>
-      <c r="J138" s="161"/>
-      <c r="K138" s="169"/>
-      <c r="L138" s="170"/>
-    </row>
-    <row r="139" spans="1:12" ht="42" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="D138" s="253" t="s">
+        <v>109</v>
+      </c>
+      <c r="E138" s="254"/>
+      <c r="F138" s="254"/>
+      <c r="G138" s="254"/>
+      <c r="H138" s="254"/>
+      <c r="I138" s="254"/>
+      <c r="J138" s="255"/>
+      <c r="K138" s="259"/>
+      <c r="L138" s="260"/>
+    </row>
+    <row r="139" spans="1:12" ht="42" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A139" s="124">
         <v>9</v>
       </c>
       <c r="B139" s="124"/>
       <c r="C139" s="126"/>
-      <c r="D139" s="159" t="s">
+      <c r="D139" s="253" t="s">
         <v>83</v>
       </c>
-      <c r="E139" s="160"/>
-      <c r="F139" s="160"/>
-      <c r="G139" s="160"/>
-      <c r="H139" s="160"/>
-      <c r="I139" s="160"/>
-      <c r="J139" s="161"/>
-      <c r="K139" s="162"/>
-      <c r="L139" s="162"/>
-    </row>
-    <row r="140" spans="1:12" ht="85.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="E139" s="254"/>
+      <c r="F139" s="254"/>
+      <c r="G139" s="254"/>
+      <c r="H139" s="254"/>
+      <c r="I139" s="254"/>
+      <c r="J139" s="255"/>
+      <c r="K139" s="226"/>
+      <c r="L139" s="226"/>
+    </row>
+    <row r="140" spans="1:12" ht="85.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A140" s="124">
         <v>10</v>
       </c>
       <c r="B140" s="124"/>
       <c r="C140" s="126"/>
-      <c r="D140" s="159" t="s">
+      <c r="D140" s="253" t="s">
         <v>84</v>
       </c>
-      <c r="E140" s="160"/>
-      <c r="F140" s="160"/>
-      <c r="G140" s="160"/>
-      <c r="H140" s="160"/>
-      <c r="I140" s="160"/>
-      <c r="J140" s="161"/>
-      <c r="K140" s="162"/>
-      <c r="L140" s="162"/>
-    </row>
-    <row r="141" spans="1:12" ht="85.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="E140" s="254"/>
+      <c r="F140" s="254"/>
+      <c r="G140" s="254"/>
+      <c r="H140" s="254"/>
+      <c r="I140" s="254"/>
+      <c r="J140" s="255"/>
+      <c r="K140" s="226"/>
+      <c r="L140" s="226"/>
+    </row>
+    <row r="141" spans="1:12" ht="85.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A141" s="124">
         <v>11</v>
       </c>
       <c r="B141" s="124"/>
       <c r="C141" s="126"/>
-      <c r="D141" s="163" t="s">
+      <c r="D141" s="256" t="s">
         <v>85</v>
       </c>
-      <c r="E141" s="164"/>
-      <c r="F141" s="164"/>
-      <c r="G141" s="164"/>
-      <c r="H141" s="164"/>
-      <c r="I141" s="164"/>
-      <c r="J141" s="165"/>
-      <c r="K141" s="162"/>
-      <c r="L141" s="162"/>
-    </row>
-    <row r="142" spans="1:12" ht="61.5" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="143" spans="1:12" ht="61.5" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="144" spans="1:12" ht="61.5" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="145" ht="61.5" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="146" ht="61.5" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="147" ht="61.5" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="148" ht="61.5" customHeight="1" x14ac:dyDescent="0.35"/>
+      <c r="E141" s="257"/>
+      <c r="F141" s="257"/>
+      <c r="G141" s="257"/>
+      <c r="H141" s="257"/>
+      <c r="I141" s="257"/>
+      <c r="J141" s="258"/>
+      <c r="K141" s="226"/>
+      <c r="L141" s="226"/>
+    </row>
+    <row r="142" spans="1:12" ht="61.5" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="143" spans="1:12" ht="61.5" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="144" spans="1:12" ht="61.5" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="145" ht="61.5" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="146" ht="61.5" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="147" ht="61.5" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="148" ht="61.5" customHeight="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <sheetProtection formatCells="0" formatColumns="0" formatRows="0"/>
   <mergeCells count="168">
-    <mergeCell ref="M2:R2"/>
-    <mergeCell ref="H18:H19"/>
-    <mergeCell ref="I18:I19"/>
-    <mergeCell ref="L15:L17"/>
-    <mergeCell ref="M15:M17"/>
-    <mergeCell ref="N15:O16"/>
-    <mergeCell ref="A1:L1"/>
-    <mergeCell ref="A2:L2"/>
-    <mergeCell ref="B15:C16"/>
-    <mergeCell ref="D15:E16"/>
-    <mergeCell ref="F15:F17"/>
-    <mergeCell ref="G15:K16"/>
-    <mergeCell ref="A4:L4"/>
-    <mergeCell ref="A5:L5"/>
-    <mergeCell ref="A6:L6"/>
-    <mergeCell ref="C9:E9"/>
-    <mergeCell ref="R15:R17"/>
-    <mergeCell ref="P15:P17"/>
-    <mergeCell ref="Q15:Q17"/>
+    <mergeCell ref="N35:O35"/>
+    <mergeCell ref="N36:O36"/>
+    <mergeCell ref="N37:O37"/>
+    <mergeCell ref="N38:O38"/>
+    <mergeCell ref="N39:O39"/>
+    <mergeCell ref="N50:O50"/>
+    <mergeCell ref="N51:O51"/>
+    <mergeCell ref="N52:O52"/>
+    <mergeCell ref="N53:O53"/>
+    <mergeCell ref="N45:O45"/>
+    <mergeCell ref="N46:O46"/>
+    <mergeCell ref="N47:O47"/>
+    <mergeCell ref="N48:O48"/>
+    <mergeCell ref="N49:O49"/>
+    <mergeCell ref="D50:E50"/>
+    <mergeCell ref="D51:E51"/>
+    <mergeCell ref="D52:E52"/>
+    <mergeCell ref="D53:E53"/>
+    <mergeCell ref="N40:O40"/>
+    <mergeCell ref="N41:O41"/>
+    <mergeCell ref="N42:O42"/>
+    <mergeCell ref="N43:O43"/>
+    <mergeCell ref="N44:O44"/>
+    <mergeCell ref="D49:E49"/>
+    <mergeCell ref="D40:E40"/>
+    <mergeCell ref="D41:E41"/>
+    <mergeCell ref="D42:E42"/>
+    <mergeCell ref="D43:E43"/>
+    <mergeCell ref="D44:E44"/>
+    <mergeCell ref="D30:E30"/>
+    <mergeCell ref="D31:E31"/>
+    <mergeCell ref="D32:E32"/>
+    <mergeCell ref="D33:E33"/>
+    <mergeCell ref="D34:E34"/>
+    <mergeCell ref="N18:O18"/>
+    <mergeCell ref="N19:O19"/>
+    <mergeCell ref="N20:O20"/>
+    <mergeCell ref="N21:O21"/>
+    <mergeCell ref="N22:O22"/>
+    <mergeCell ref="N23:O23"/>
+    <mergeCell ref="N24:O24"/>
+    <mergeCell ref="N25:O25"/>
+    <mergeCell ref="N26:O26"/>
+    <mergeCell ref="N30:O30"/>
+    <mergeCell ref="N31:O31"/>
+    <mergeCell ref="N32:O32"/>
+    <mergeCell ref="N33:O33"/>
+    <mergeCell ref="N34:O34"/>
+    <mergeCell ref="D35:E35"/>
+    <mergeCell ref="D36:E36"/>
+    <mergeCell ref="D37:E37"/>
+    <mergeCell ref="D38:E38"/>
+    <mergeCell ref="D39:E39"/>
+    <mergeCell ref="D140:J140"/>
+    <mergeCell ref="K140:L140"/>
+    <mergeCell ref="D141:J141"/>
+    <mergeCell ref="K141:L141"/>
+    <mergeCell ref="D137:J137"/>
+    <mergeCell ref="K137:L137"/>
+    <mergeCell ref="D138:J138"/>
+    <mergeCell ref="K138:L138"/>
+    <mergeCell ref="D139:J139"/>
+    <mergeCell ref="K139:L139"/>
+    <mergeCell ref="D134:J134"/>
+    <mergeCell ref="K134:L134"/>
+    <mergeCell ref="D135:J135"/>
+    <mergeCell ref="K135:L135"/>
+    <mergeCell ref="D136:J136"/>
+    <mergeCell ref="K136:L136"/>
+    <mergeCell ref="D131:J131"/>
+    <mergeCell ref="K131:L131"/>
+    <mergeCell ref="D132:J132"/>
+    <mergeCell ref="K132:L132"/>
+    <mergeCell ref="D133:J133"/>
+    <mergeCell ref="K133:L133"/>
+    <mergeCell ref="B129:C129"/>
+    <mergeCell ref="D129:J130"/>
+    <mergeCell ref="K129:L130"/>
+    <mergeCell ref="F88:J88"/>
+    <mergeCell ref="M88:R88"/>
+    <mergeCell ref="M95:R95"/>
+    <mergeCell ref="M96:R96"/>
+    <mergeCell ref="M97:R97"/>
+    <mergeCell ref="M98:R98"/>
+    <mergeCell ref="M99:R99"/>
+    <mergeCell ref="A124:L124"/>
+    <mergeCell ref="A125:L125"/>
+    <mergeCell ref="D126:I126"/>
+    <mergeCell ref="J126:L126"/>
+    <mergeCell ref="M87:R87"/>
+    <mergeCell ref="M73:R73"/>
+    <mergeCell ref="F75:K75"/>
+    <mergeCell ref="M75:R75"/>
+    <mergeCell ref="F77:J77"/>
+    <mergeCell ref="P79:Q79"/>
+    <mergeCell ref="O78:R78"/>
+    <mergeCell ref="O81:R81"/>
+    <mergeCell ref="M83:R83"/>
+    <mergeCell ref="M84:R84"/>
+    <mergeCell ref="M85:R85"/>
+    <mergeCell ref="M86:R86"/>
+    <mergeCell ref="M72:R72"/>
+    <mergeCell ref="B40:C41"/>
+    <mergeCell ref="B42:C43"/>
+    <mergeCell ref="B44:C45"/>
+    <mergeCell ref="B46:C47"/>
+    <mergeCell ref="B48:C49"/>
+    <mergeCell ref="B50:C51"/>
+    <mergeCell ref="Q18:Q53"/>
+    <mergeCell ref="B52:C53"/>
+    <mergeCell ref="G58:H58"/>
+    <mergeCell ref="G59:H59"/>
+    <mergeCell ref="C63:K64"/>
+    <mergeCell ref="M71:R71"/>
+    <mergeCell ref="B28:C29"/>
+    <mergeCell ref="B30:C31"/>
+    <mergeCell ref="B32:C33"/>
+    <mergeCell ref="B34:C35"/>
+    <mergeCell ref="B36:C37"/>
+    <mergeCell ref="D25:E25"/>
+    <mergeCell ref="D26:E26"/>
+    <mergeCell ref="D27:E27"/>
+    <mergeCell ref="D28:E28"/>
+    <mergeCell ref="D29:E29"/>
+    <mergeCell ref="D20:E20"/>
     <mergeCell ref="B38:C39"/>
     <mergeCell ref="J18:J19"/>
     <mergeCell ref="K18:K19"/>
@@ -6123,131 +6185,25 @@
     <mergeCell ref="D46:E46"/>
     <mergeCell ref="D47:E47"/>
     <mergeCell ref="D48:E48"/>
-    <mergeCell ref="M72:R72"/>
-    <mergeCell ref="B40:C41"/>
-    <mergeCell ref="B42:C43"/>
-    <mergeCell ref="B44:C45"/>
-    <mergeCell ref="B46:C47"/>
-    <mergeCell ref="B48:C49"/>
-    <mergeCell ref="B50:C51"/>
-    <mergeCell ref="Q18:Q53"/>
-    <mergeCell ref="B52:C53"/>
-    <mergeCell ref="G58:H58"/>
-    <mergeCell ref="G59:H59"/>
-    <mergeCell ref="C63:K64"/>
-    <mergeCell ref="M71:R71"/>
-    <mergeCell ref="B28:C29"/>
-    <mergeCell ref="B30:C31"/>
-    <mergeCell ref="B32:C33"/>
-    <mergeCell ref="B34:C35"/>
-    <mergeCell ref="B36:C37"/>
-    <mergeCell ref="D25:E25"/>
-    <mergeCell ref="D26:E26"/>
-    <mergeCell ref="D27:E27"/>
-    <mergeCell ref="D28:E28"/>
-    <mergeCell ref="D29:E29"/>
-    <mergeCell ref="D20:E20"/>
-    <mergeCell ref="M87:R87"/>
-    <mergeCell ref="M73:R73"/>
-    <mergeCell ref="F75:K75"/>
-    <mergeCell ref="M75:R75"/>
-    <mergeCell ref="F77:J77"/>
-    <mergeCell ref="P79:Q79"/>
-    <mergeCell ref="O78:R78"/>
-    <mergeCell ref="O81:R81"/>
-    <mergeCell ref="M83:R83"/>
-    <mergeCell ref="M84:R84"/>
-    <mergeCell ref="M85:R85"/>
-    <mergeCell ref="M86:R86"/>
-    <mergeCell ref="K132:L132"/>
-    <mergeCell ref="D133:J133"/>
-    <mergeCell ref="K133:L133"/>
-    <mergeCell ref="B129:C129"/>
-    <mergeCell ref="D129:J130"/>
-    <mergeCell ref="K129:L130"/>
-    <mergeCell ref="F88:J88"/>
-    <mergeCell ref="M88:R88"/>
-    <mergeCell ref="M95:R95"/>
-    <mergeCell ref="M96:R96"/>
-    <mergeCell ref="M97:R97"/>
-    <mergeCell ref="M98:R98"/>
-    <mergeCell ref="M99:R99"/>
-    <mergeCell ref="A124:L124"/>
-    <mergeCell ref="A125:L125"/>
-    <mergeCell ref="D126:I126"/>
-    <mergeCell ref="J126:L126"/>
-    <mergeCell ref="D35:E35"/>
-    <mergeCell ref="D36:E36"/>
-    <mergeCell ref="D37:E37"/>
-    <mergeCell ref="D38:E38"/>
-    <mergeCell ref="D39:E39"/>
-    <mergeCell ref="D140:J140"/>
-    <mergeCell ref="K140:L140"/>
-    <mergeCell ref="D141:J141"/>
-    <mergeCell ref="K141:L141"/>
-    <mergeCell ref="D137:J137"/>
-    <mergeCell ref="K137:L137"/>
-    <mergeCell ref="D138:J138"/>
-    <mergeCell ref="K138:L138"/>
-    <mergeCell ref="D139:J139"/>
-    <mergeCell ref="K139:L139"/>
-    <mergeCell ref="D134:J134"/>
-    <mergeCell ref="K134:L134"/>
-    <mergeCell ref="D135:J135"/>
-    <mergeCell ref="K135:L135"/>
-    <mergeCell ref="D136:J136"/>
-    <mergeCell ref="K136:L136"/>
-    <mergeCell ref="D131:J131"/>
-    <mergeCell ref="K131:L131"/>
-    <mergeCell ref="D132:J132"/>
-    <mergeCell ref="D30:E30"/>
-    <mergeCell ref="D31:E31"/>
-    <mergeCell ref="D32:E32"/>
-    <mergeCell ref="D33:E33"/>
-    <mergeCell ref="D34:E34"/>
-    <mergeCell ref="N18:O18"/>
-    <mergeCell ref="N19:O19"/>
-    <mergeCell ref="N20:O20"/>
-    <mergeCell ref="N21:O21"/>
-    <mergeCell ref="N22:O22"/>
-    <mergeCell ref="N23:O23"/>
-    <mergeCell ref="N24:O24"/>
-    <mergeCell ref="N25:O25"/>
-    <mergeCell ref="N26:O26"/>
-    <mergeCell ref="N30:O30"/>
-    <mergeCell ref="N31:O31"/>
-    <mergeCell ref="N32:O32"/>
-    <mergeCell ref="N33:O33"/>
-    <mergeCell ref="N34:O34"/>
-    <mergeCell ref="D50:E50"/>
-    <mergeCell ref="D51:E51"/>
-    <mergeCell ref="D52:E52"/>
-    <mergeCell ref="D53:E53"/>
-    <mergeCell ref="N40:O40"/>
-    <mergeCell ref="N41:O41"/>
-    <mergeCell ref="N42:O42"/>
-    <mergeCell ref="N43:O43"/>
-    <mergeCell ref="N44:O44"/>
-    <mergeCell ref="D49:E49"/>
-    <mergeCell ref="D40:E40"/>
-    <mergeCell ref="D41:E41"/>
-    <mergeCell ref="D42:E42"/>
-    <mergeCell ref="D43:E43"/>
-    <mergeCell ref="D44:E44"/>
-    <mergeCell ref="N35:O35"/>
-    <mergeCell ref="N36:O36"/>
-    <mergeCell ref="N37:O37"/>
-    <mergeCell ref="N38:O38"/>
-    <mergeCell ref="N39:O39"/>
-    <mergeCell ref="N50:O50"/>
-    <mergeCell ref="N51:O51"/>
-    <mergeCell ref="N52:O52"/>
-    <mergeCell ref="N53:O53"/>
-    <mergeCell ref="N45:O45"/>
-    <mergeCell ref="N46:O46"/>
-    <mergeCell ref="N47:O47"/>
-    <mergeCell ref="N48:O48"/>
-    <mergeCell ref="N49:O49"/>
+    <mergeCell ref="M2:R2"/>
+    <mergeCell ref="H18:H19"/>
+    <mergeCell ref="I18:I19"/>
+    <mergeCell ref="L15:L17"/>
+    <mergeCell ref="M15:M17"/>
+    <mergeCell ref="N15:O16"/>
+    <mergeCell ref="A1:L1"/>
+    <mergeCell ref="A2:L2"/>
+    <mergeCell ref="B15:C16"/>
+    <mergeCell ref="D15:E16"/>
+    <mergeCell ref="F15:F17"/>
+    <mergeCell ref="G15:K16"/>
+    <mergeCell ref="A4:L4"/>
+    <mergeCell ref="A5:L5"/>
+    <mergeCell ref="A6:L6"/>
+    <mergeCell ref="C9:E9"/>
+    <mergeCell ref="R15:R17"/>
+    <mergeCell ref="P15:P17"/>
+    <mergeCell ref="Q15:Q17"/>
   </mergeCells>
   <phoneticPr fontId="40" type="noConversion"/>
   <printOptions horizontalCentered="1"/>

</xml_diff>